<commit_message>
📊 BIST Screener | 19.05.2026 08:30 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-19.xlsx
+++ b/data/bist_screener_2026-05-19.xlsx
@@ -25909,23 +25909,21 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>30.64</v>
+        <v>178.6</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.07820000000000001</v>
+        <v>-0.0341</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>16140000</v>
-      </c>
-      <c r="E587" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>8620000</v>
+      </c>
+      <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>52.53</v>
+        <v>38.77</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25938,7 +25936,7 @@
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25946,38 +25944,34 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>65.15000000000001</v>
+        <v>198.4</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0585</v>
+        <v>-0.0345</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>869750</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>8520000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>49.58</v>
+        <v>61.52</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="4" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25985,21 +25979,23 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>13.96</v>
+        <v>30.64</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0285</v>
+        <v>-0.07820000000000001</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>30370000</v>
-      </c>
-      <c r="E589" s="6" t="inlineStr"/>
+        <v>16140000</v>
+      </c>
+      <c r="E589" s="8" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F589" s="7" t="n">
-        <v>49.07</v>
+        <v>52.53</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26007,12 +26003,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26020,147 +26016,149 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>142.7</v>
+        <v>9.93</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.061</v>
+        <v>0.0793</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>995180</v>
+        <v>757940</v>
       </c>
       <c r="E590" s="4" t="n">
-        <v>0.1071</v>
+        <v>0.95</v>
       </c>
       <c r="F590" s="3" t="n">
-        <v>48.18</v>
+        <v>61.27</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="4" t="n">
-        <v>-3.6635</v>
+        <v>-23.6291</v>
       </c>
       <c r="J590" s="4" t="n">
-        <v>-0.4897</v>
+        <v>-0.4678</v>
       </c>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
-        </is>
-      </c>
-      <c r="L590" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr"/>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>36.4</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0196</v>
+        <v>0.0162</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>6480000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>48030</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>58.24</v>
+        <v>36.59</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="6" t="inlineStr"/>
+      <c r="I591" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J591" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr"/>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>69.09999999999999</v>
+        <v>28.4</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0162</v>
+        <v>-0.0373</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>48030</v>
-      </c>
-      <c r="E592" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>23640000</v>
+      </c>
+      <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>36.59</v>
+        <v>55.6</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J592" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I592" s="2" t="inlineStr"/>
+      <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr"/>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr">
+        <is>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>198.4</v>
+        <v>5.97</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0345</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>8520000</v>
-      </c>
-      <c r="E593" s="6" t="inlineStr"/>
+        <v>35800000</v>
+      </c>
+      <c r="E593" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F593" s="7" t="n">
-        <v>61.52</v>
+        <v>49.23</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="6" t="inlineStr"/>
+      <c r="I593" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J593" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26168,23 +26166,21 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>6.44</v>
+        <v>6.06</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0733</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>19120000</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>7340000</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>70.31</v>
+        <v>45.24</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26195,31 +26191,27 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L594" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
-        </is>
-      </c>
+      <c r="L594" s="2" t="inlineStr"/>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>178.6</v>
+        <v>13.96</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0341</v>
+        <v>-0.0285</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>8620000</v>
+        <v>30370000</v>
       </c>
       <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>38.77</v>
+        <v>49.07</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
@@ -26227,12 +26219,12 @@
       <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26240,21 +26232,21 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>42.32</v>
+        <v>17.05</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0272</v>
+        <v>-0.0512</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>5980000</v>
+        <v>48680000</v>
       </c>
       <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>53.18</v>
+        <v>49.01</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26262,12 +26254,12 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26275,21 +26267,21 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>6.06</v>
+        <v>2.73</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.008199999999999999</v>
+        <v>0</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>7340000</v>
+        <v>142720000</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>45.24</v>
+        <v>45.93</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26300,40 +26292,48 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L597" s="6" t="inlineStr"/>
+      <c r="L597" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>17.05</v>
+        <v>65.15000000000001</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0512</v>
+        <v>-0.0585</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>48680000</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>869750</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>49.01</v>
+        <v>49.58</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="2" t="inlineStr"/>
+      <c r="J598" s="4" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26341,81 +26341,67 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>34.68</v>
+        <v>78.62</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0181</v>
+        <v>-0.0067</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>5190000</v>
-      </c>
-      <c r="E599" s="8" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>11350000</v>
+      </c>
+      <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>43.26</v>
-      </c>
-      <c r="G599" s="7" t="n">
-        <v>13.71</v>
-      </c>
+        <v>37.39</v>
+      </c>
+      <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
-      <c r="I599" s="8" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J599" s="8" t="n">
-        <v>-1.4864</v>
-      </c>
-      <c r="K599" s="6" t="inlineStr">
-        <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+      <c r="I599" s="6" t="inlineStr"/>
+      <c r="J599" s="6" t="inlineStr"/>
+      <c r="K599" s="6" t="inlineStr"/>
+      <c r="L599" s="6" t="inlineStr"/>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>26.02</v>
+        <v>2.48</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.008399999999999999</v>
+        <v>-0.008</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>883760</v>
+        <v>21880000</v>
       </c>
       <c r="E600" s="4" t="n">
-        <v>0.9698</v>
+        <v>1</v>
       </c>
       <c r="F600" s="3" t="n">
-        <v>43.34</v>
+        <v>35.12</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="2" t="inlineStr"/>
+      <c r="I600" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
       <c r="J600" s="4" t="n">
-        <v>0.6453</v>
+        <v>-0.8093</v>
       </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26423,40 +26409,34 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>2.48</v>
+        <v>18.53</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.008</v>
+        <v>0.0011</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>21880000</v>
-      </c>
-      <c r="E601" s="8" t="n">
-        <v>1</v>
-      </c>
+        <v>55440000</v>
+      </c>
+      <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>35.12</v>
+        <v>35.89</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J601" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26464,34 +26444,40 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>28.4</v>
+        <v>142.7</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0373</v>
+        <v>0.061</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>23640000</v>
-      </c>
-      <c r="E602" s="2" t="inlineStr"/>
+        <v>995180</v>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F602" s="3" t="n">
-        <v>55.6</v>
+        <v>48.18</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="2" t="inlineStr"/>
-      <c r="J602" s="2" t="inlineStr"/>
+      <c r="I602" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J602" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26534,50 +26520,56 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>78.62</v>
+        <v>36.4</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0067</v>
+        <v>0.0196</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>11350000</v>
+        <v>6480000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>37.39</v>
+        <v>58.24</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
       <c r="I604" s="2" t="inlineStr"/>
       <c r="J604" s="2" t="inlineStr"/>
-      <c r="K604" s="2" t="inlineStr"/>
-      <c r="L604" s="2" t="inlineStr"/>
+      <c r="K604" s="2" t="inlineStr">
+        <is>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>240.1</v>
+        <v>73.8</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.02</v>
+        <v>-0.0238</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>10620</v>
-      </c>
-      <c r="E605" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>174630</v>
+      </c>
+      <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>43.77</v>
+        <v>10.48</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26585,7 +26577,7 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr"/>
@@ -26594,77 +26586,77 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>9.93</v>
+        <v>42.32</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0793</v>
+        <v>0.0272</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>757940</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>0.95</v>
-      </c>
+        <v>5980000</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>61.27</v>
+        <v>53.18</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J606" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I606" s="2" t="inlineStr"/>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>5.97</v>
+        <v>34.68</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.09939999999999999</v>
+        <v>-0.0181</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>35800000</v>
+        <v>5190000</v>
       </c>
       <c r="E607" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.3528</v>
       </c>
       <c r="F607" s="7" t="n">
-        <v>49.23</v>
-      </c>
-      <c r="G607" s="6" t="inlineStr"/>
+        <v>43.26</v>
+      </c>
+      <c r="G607" s="7" t="n">
+        <v>13.71</v>
+      </c>
       <c r="H607" s="6" t="inlineStr"/>
       <c r="I607" s="8" t="n">
-        <v>-5.3262</v>
+        <v>0.1029</v>
       </c>
       <c r="J607" s="8" t="n">
-        <v>-4.2562</v>
+        <v>-1.4864</v>
       </c>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26672,21 +26664,21 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>2.73</v>
+        <v>77.25</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>142720000</v>
+        <v>29900000</v>
       </c>
       <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>45.93</v>
+        <v>88.89</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
@@ -26694,12 +26686,12 @@
       <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26707,21 +26699,23 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>77.25</v>
+        <v>240.1</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.09960000000000001</v>
+        <v>-0.02</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>29900000</v>
-      </c>
-      <c r="E609" s="6" t="inlineStr"/>
+        <v>10620</v>
+      </c>
+      <c r="E609" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F609" s="7" t="n">
-        <v>88.89</v>
+        <v>43.77</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
@@ -26729,47 +26723,47 @@
       <c r="J609" s="6" t="inlineStr"/>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L609" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L609" s="6" t="inlineStr"/>
       <c r="M609" s="6" t="inlineStr"/>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>18.53</v>
+        <v>26.02</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>0.0011</v>
+        <v>-0.008399999999999999</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>55440000</v>
-      </c>
-      <c r="E610" s="2" t="inlineStr"/>
+        <v>883760</v>
+      </c>
+      <c r="E610" s="4" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F610" s="3" t="n">
-        <v>35.89</v>
+        <v>43.34</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
       <c r="I610" s="2" t="inlineStr"/>
-      <c r="J610" s="2" t="inlineStr"/>
+      <c r="J610" s="4" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M610" s="2" t="inlineStr"/>
@@ -26777,21 +26771,23 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>73.8</v>
+        <v>6.44</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.0238</v>
+        <v>0.0733</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>174630</v>
-      </c>
-      <c r="E611" s="6" t="inlineStr"/>
+        <v>19120000</v>
+      </c>
+      <c r="E611" s="8" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F611" s="7" t="n">
-        <v>10.48</v>
+        <v>70.31</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
@@ -26802,7 +26798,11 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L611" s="6" t="inlineStr"/>
+      <c r="L611" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M611" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26827,7 +26827,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>19.05.2026 07:30</t>
+          <t>19.05.2026 08:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 19.05.2026 09:30 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-19.xlsx
+++ b/data/bist_screener_2026-05-19.xlsx
@@ -25909,21 +25909,21 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>178.6</v>
+        <v>2.73</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.0341</v>
+        <v>0</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>8620000</v>
+        <v>142720000</v>
       </c>
       <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>38.77</v>
+        <v>45.93</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25931,12 +25931,12 @@
       <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25944,21 +25944,21 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>198.4</v>
+        <v>13.96</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0345</v>
+        <v>-0.0285</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>8520000</v>
+        <v>30370000</v>
       </c>
       <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>61.52</v>
+        <v>49.07</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25966,12 +25966,12 @@
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25979,23 +25979,23 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>30.64</v>
+        <v>6.44</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.07820000000000001</v>
+        <v>0.0733</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>16140000</v>
+        <v>19120000</v>
       </c>
       <c r="E589" s="8" t="n">
-        <v>0.2667</v>
+        <v>0.8667</v>
       </c>
       <c r="F589" s="7" t="n">
-        <v>52.53</v>
+        <v>70.31</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26003,12 +26003,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26016,108 +26016,114 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>9.93</v>
+        <v>2.48</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0793</v>
+        <v>-0.008</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>757940</v>
+        <v>21880000</v>
       </c>
       <c r="E590" s="4" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="F590" s="3" t="n">
-        <v>61.27</v>
+        <v>35.12</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="4" t="n">
-        <v>-23.6291</v>
+        <v>-191.6342</v>
       </c>
       <c r="J590" s="4" t="n">
-        <v>-0.4678</v>
+        <v>-0.8093</v>
       </c>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L590" s="2" t="inlineStr"/>
+          <t>Dağıtım servisleri</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>69.09999999999999</v>
+        <v>198.4</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0162</v>
+        <v>-0.0345</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>48030</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.58</v>
-      </c>
+        <v>8520000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>36.59</v>
+        <v>61.52</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J591" s="8" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I591" s="6" t="inlineStr"/>
+      <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>28.4</v>
+        <v>26.02</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0373</v>
+        <v>-0.008399999999999999</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>23640000</v>
-      </c>
-      <c r="E592" s="2" t="inlineStr"/>
+        <v>883760</v>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F592" s="3" t="n">
-        <v>55.6</v>
+        <v>43.34</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
       <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="2" t="inlineStr"/>
+      <c r="J592" s="4" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26125,40 +26131,34 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>5.97</v>
+        <v>42.32</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.09939999999999999</v>
+        <v>0.0272</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>35800000</v>
-      </c>
-      <c r="E593" s="8" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>5980000</v>
+      </c>
+      <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>49.23</v>
+        <v>53.18</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J593" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I593" s="6" t="inlineStr"/>
+      <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26166,21 +26166,21 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>6.06</v>
+        <v>17.05</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.008199999999999999</v>
+        <v>-0.0512</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>7340000</v>
+        <v>48680000</v>
       </c>
       <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>45.24</v>
+        <v>49.01</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26191,40 +26191,50 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L594" s="2" t="inlineStr"/>
+      <c r="L594" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>13.96</v>
+        <v>142.7</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0285</v>
+        <v>0.061</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>30370000</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
+        <v>995180</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F595" s="7" t="n">
-        <v>49.07</v>
+        <v>48.18</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="6" t="inlineStr"/>
+      <c r="I595" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J595" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26232,21 +26242,23 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>17.05</v>
+        <v>30.64</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0512</v>
+        <v>-0.07820000000000001</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>48680000</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>16140000</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>49.01</v>
+        <v>52.53</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26254,12 +26266,12 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26267,21 +26279,21 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>2.73</v>
+        <v>18.53</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0</v>
+        <v>0.0011</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>142720000</v>
+        <v>55440000</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>45.93</v>
+        <v>35.89</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26294,7 +26306,7 @@
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26341,67 +26353,69 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>78.62</v>
+        <v>77.25</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0067</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>11350000</v>
+        <v>29900000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>37.39</v>
+        <v>88.89</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
       <c r="I599" s="6" t="inlineStr"/>
       <c r="J599" s="6" t="inlineStr"/>
-      <c r="K599" s="6" t="inlineStr"/>
-      <c r="L599" s="6" t="inlineStr"/>
+      <c r="K599" s="6" t="inlineStr">
+        <is>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>2.48</v>
+        <v>36.4</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.008</v>
+        <v>0.0196</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>21880000</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>6480000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>35.12</v>
+        <v>58.24</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J600" s="4" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I600" s="2" t="inlineStr"/>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26409,21 +26423,21 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>18.53</v>
+        <v>28.4</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0011</v>
+        <v>-0.0373</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>55440000</v>
+        <v>23640000</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>35.89</v>
+        <v>55.6</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
@@ -26431,12 +26445,12 @@
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26444,40 +26458,34 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>142.7</v>
+        <v>18.16</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.061</v>
+        <v>0.0145</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>995180</v>
-      </c>
-      <c r="E602" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>45490000</v>
+      </c>
+      <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>48.18</v>
+        <v>52.57</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J602" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I602" s="2" t="inlineStr"/>
+      <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26485,91 +26493,87 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>18.16</v>
+        <v>9.93</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0145</v>
+        <v>0.0793</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>45490000</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>757940</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>52.57</v>
+        <v>61.27</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="6" t="inlineStr"/>
+      <c r="I603" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J603" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr"/>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>36.4</v>
+        <v>78.62</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0196</v>
+        <v>-0.0067</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>6480000</v>
+        <v>11350000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>58.24</v>
+        <v>37.39</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
       <c r="I604" s="2" t="inlineStr"/>
       <c r="J604" s="2" t="inlineStr"/>
-      <c r="K604" s="2" t="inlineStr">
-        <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+      <c r="K604" s="2" t="inlineStr"/>
+      <c r="L604" s="2" t="inlineStr"/>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>73.8</v>
+        <v>240.1</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.0238</v>
+        <v>-0.02</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>174630</v>
-      </c>
-      <c r="E605" s="6" t="inlineStr"/>
+        <v>10620</v>
+      </c>
+      <c r="E605" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F605" s="7" t="n">
-        <v>10.48</v>
+        <v>43.77</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26577,7 +26581,7 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr"/>
@@ -26586,21 +26590,21 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>42.32</v>
+        <v>178.6</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0272</v>
+        <v>-0.0341</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>5980000</v>
+        <v>8620000</v>
       </c>
       <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>53.18</v>
+        <v>38.77</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26608,12 +26612,12 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26621,42 +26625,40 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>34.68</v>
+        <v>5.97</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0181</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>5190000</v>
+        <v>35800000</v>
       </c>
       <c r="E607" s="8" t="n">
-        <v>0.3528</v>
+        <v>0.1672</v>
       </c>
       <c r="F607" s="7" t="n">
-        <v>43.26</v>
-      </c>
-      <c r="G607" s="7" t="n">
-        <v>13.71</v>
-      </c>
+        <v>49.23</v>
+      </c>
+      <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
       <c r="I607" s="8" t="n">
-        <v>0.1029</v>
+        <v>-5.3262</v>
       </c>
       <c r="J607" s="8" t="n">
-        <v>-1.4864</v>
+        <v>-4.2562</v>
       </c>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26664,21 +26666,21 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>77.25</v>
+        <v>6.06</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.09960000000000001</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>29900000</v>
+        <v>7340000</v>
       </c>
       <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>88.89</v>
+        <v>45.24</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
@@ -26686,36 +26688,30 @@
       <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L608" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L608" s="2" t="inlineStr"/>
       <c r="M608" s="2" t="inlineStr"/>
     </row>
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>240.1</v>
+        <v>73.8</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>-0.02</v>
+        <v>-0.0238</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>10620</v>
-      </c>
-      <c r="E609" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>174630</v>
+      </c>
+      <c r="E609" s="6" t="inlineStr"/>
       <c r="F609" s="7" t="n">
-        <v>43.77</v>
+        <v>10.48</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
@@ -26723,7 +26719,7 @@
       <c r="J609" s="6" t="inlineStr"/>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr"/>
@@ -26732,29 +26728,33 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>26.02</v>
+        <v>34.68</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.008399999999999999</v>
+        <v>-0.0181</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>883760</v>
+        <v>5190000</v>
       </c>
       <c r="E610" s="4" t="n">
-        <v>0.9698</v>
+        <v>0.3528</v>
       </c>
       <c r="F610" s="3" t="n">
-        <v>43.34</v>
-      </c>
-      <c r="G610" s="2" t="inlineStr"/>
+        <v>43.26</v>
+      </c>
+      <c r="G610" s="3" t="n">
+        <v>13.71</v>
+      </c>
       <c r="H610" s="2" t="inlineStr"/>
-      <c r="I610" s="2" t="inlineStr"/>
+      <c r="I610" s="4" t="n">
+        <v>0.1029</v>
+      </c>
       <c r="J610" s="4" t="n">
-        <v>0.6453</v>
+        <v>-1.4864</v>
       </c>
       <c r="K610" s="2" t="inlineStr">
         <is>
@@ -26763,7 +26763,7 @@
       </c>
       <c r="L610" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M610" s="2" t="inlineStr"/>
@@ -26771,38 +26771,38 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>6.44</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>0.0733</v>
+        <v>0.0162</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>19120000</v>
+        <v>48030</v>
       </c>
       <c r="E611" s="8" t="n">
-        <v>0.8667</v>
+        <v>0.58</v>
       </c>
       <c r="F611" s="7" t="n">
-        <v>70.31</v>
+        <v>36.59</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="6" t="inlineStr"/>
-      <c r="J611" s="6" t="inlineStr"/>
+      <c r="I611" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J611" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L611" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L611" s="6" t="inlineStr"/>
       <c r="M611" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26827,7 +26827,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>19.05.2026 08:30</t>
+          <t>19.05.2026 09:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 19.05.2026 10:30 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-19.xlsx
+++ b/data/bist_screener_2026-05-19.xlsx
@@ -15811,40 +15811,44 @@
     <row r="353">
       <c r="A353" s="6" t="inlineStr">
         <is>
-          <t>HURGZ</t>
+          <t>OFSYM</t>
         </is>
       </c>
       <c r="B353" s="7" t="n">
-        <v>8.77</v>
+        <v>57.7</v>
       </c>
       <c r="C353" s="8" t="n">
-        <v>-0.0201</v>
+        <v>0.0009</v>
       </c>
       <c r="D353" s="9" t="n">
-        <v>27210000</v>
+        <v>2440000</v>
       </c>
       <c r="E353" s="8" t="n">
-        <v>0.1879</v>
+        <v>0.1556</v>
       </c>
       <c r="F353" s="7" t="n">
-        <v>62.4</v>
-      </c>
-      <c r="G353" s="6" t="inlineStr"/>
+        <v>43.19</v>
+      </c>
+      <c r="G353" s="7" t="n">
+        <v>28.65</v>
+      </c>
       <c r="H353" s="7" t="n">
         <v>2.05</v>
       </c>
       <c r="I353" s="8" t="n">
-        <v>-0.3044</v>
-      </c>
-      <c r="J353" s="6" t="inlineStr"/>
+        <v>0.08449999999999999</v>
+      </c>
+      <c r="J353" s="8" t="n">
+        <v>0.1882</v>
+      </c>
       <c r="K353" s="6" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L353" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST ANKARA</t>
         </is>
       </c>
       <c r="M353" s="6" t="inlineStr"/>
@@ -15852,44 +15856,42 @@
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>OFSYM</t>
+          <t>HUBVC</t>
         </is>
       </c>
       <c r="B354" s="3" t="n">
-        <v>57.7</v>
+        <v>3.84</v>
       </c>
       <c r="C354" s="4" t="n">
-        <v>0.0009</v>
+        <v>-0.0278</v>
       </c>
       <c r="D354" s="5" t="n">
-        <v>2440000</v>
+        <v>2960000</v>
       </c>
       <c r="E354" s="4" t="n">
-        <v>0.1556</v>
+        <v>0.8462000000000001</v>
       </c>
       <c r="F354" s="3" t="n">
-        <v>43.19</v>
-      </c>
-      <c r="G354" s="3" t="n">
-        <v>28.65</v>
-      </c>
+        <v>49.06</v>
+      </c>
+      <c r="G354" s="2" t="inlineStr"/>
       <c r="H354" s="3" t="n">
         <v>2.05</v>
       </c>
       <c r="I354" s="4" t="n">
-        <v>0.08449999999999999</v>
+        <v>-0.9107</v>
       </c>
       <c r="J354" s="4" t="n">
-        <v>0.1882</v>
+        <v>-3.7217</v>
       </c>
       <c r="K354" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L354" s="2" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST ANKARA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST MALİ</t>
         </is>
       </c>
       <c r="M354" s="2" t="inlineStr"/>
@@ -15897,42 +15899,44 @@
     <row r="355">
       <c r="A355" s="6" t="inlineStr">
         <is>
-          <t>HUBVC</t>
+          <t>BEYAZ</t>
         </is>
       </c>
       <c r="B355" s="7" t="n">
-        <v>3.84</v>
+        <v>28.12</v>
       </c>
       <c r="C355" s="8" t="n">
-        <v>-0.0278</v>
+        <v>-0.035</v>
       </c>
       <c r="D355" s="9" t="n">
-        <v>2960000</v>
+        <v>1300000</v>
       </c>
       <c r="E355" s="8" t="n">
-        <v>0.8462000000000001</v>
+        <v>0.2455</v>
       </c>
       <c r="F355" s="7" t="n">
-        <v>49.06</v>
-      </c>
-      <c r="G355" s="6" t="inlineStr"/>
+        <v>39.39</v>
+      </c>
+      <c r="G355" s="7" t="n">
+        <v>22</v>
+      </c>
       <c r="H355" s="7" t="n">
-        <v>2.05</v>
+        <v>2.1</v>
       </c>
       <c r="I355" s="8" t="n">
-        <v>-0.9107</v>
+        <v>0.1128</v>
       </c>
       <c r="J355" s="8" t="n">
-        <v>-3.7217</v>
+        <v>-0.9066</v>
       </c>
       <c r="K355" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L355" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST MALİ</t>
+          <t>BIST ULASTIRMA, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST ANA, BIST BALIKESİR</t>
         </is>
       </c>
       <c r="M355" s="6" t="inlineStr"/>
@@ -15940,44 +15944,44 @@
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>BEYAZ</t>
+          <t>EGPRO</t>
         </is>
       </c>
       <c r="B356" s="3" t="n">
-        <v>28.12</v>
+        <v>38.98</v>
       </c>
       <c r="C356" s="4" t="n">
-        <v>-0.035</v>
+        <v>-0.0231</v>
       </c>
       <c r="D356" s="5" t="n">
-        <v>1300000</v>
+        <v>2120000</v>
       </c>
       <c r="E356" s="4" t="n">
-        <v>0.2455</v>
+        <v>0.1314</v>
       </c>
       <c r="F356" s="3" t="n">
-        <v>39.39</v>
+        <v>49.98</v>
       </c>
       <c r="G356" s="3" t="n">
-        <v>22</v>
+        <v>17.42</v>
       </c>
       <c r="H356" s="3" t="n">
-        <v>2.1</v>
+        <v>2.11</v>
       </c>
       <c r="I356" s="4" t="n">
-        <v>0.1128</v>
+        <v>0.1433</v>
       </c>
       <c r="J356" s="4" t="n">
-        <v>-0.9066</v>
+        <v>-0.2049</v>
       </c>
       <c r="K356" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L356" s="2" t="inlineStr">
         <is>
-          <t>BIST ULASTIRMA, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST ANA, BIST BALIKESİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU, BIST İZMİR</t>
         </is>
       </c>
       <c r="M356" s="2" t="inlineStr"/>
@@ -15985,44 +15989,40 @@
     <row r="357">
       <c r="A357" s="6" t="inlineStr">
         <is>
-          <t>EGPRO</t>
+          <t>ZGYO</t>
         </is>
       </c>
       <c r="B357" s="7" t="n">
-        <v>38.98</v>
+        <v>31.78</v>
       </c>
       <c r="C357" s="8" t="n">
-        <v>-0.0231</v>
+        <v>-0.013</v>
       </c>
       <c r="D357" s="9" t="n">
-        <v>2120000</v>
+        <v>10400000</v>
       </c>
       <c r="E357" s="8" t="n">
-        <v>0.1314</v>
+        <v>0.2007</v>
       </c>
       <c r="F357" s="7" t="n">
-        <v>49.98</v>
-      </c>
-      <c r="G357" s="7" t="n">
-        <v>17.42</v>
-      </c>
+        <v>55.33</v>
+      </c>
+      <c r="G357" s="6" t="inlineStr"/>
       <c r="H357" s="7" t="n">
-        <v>2.11</v>
-      </c>
-      <c r="I357" s="8" t="n">
-        <v>0.1433</v>
-      </c>
+        <v>2.12</v>
+      </c>
+      <c r="I357" s="6" t="inlineStr"/>
       <c r="J357" s="8" t="n">
-        <v>-0.2049</v>
+        <v>-0.8944</v>
       </c>
       <c r="K357" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L357" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M357" s="6" t="inlineStr"/>
@@ -16030,40 +16030,42 @@
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>ZGYO</t>
+          <t>SONME</t>
         </is>
       </c>
       <c r="B358" s="3" t="n">
-        <v>31.78</v>
+        <v>134.3</v>
       </c>
       <c r="C358" s="4" t="n">
-        <v>-0.013</v>
+        <v>-0.0118</v>
       </c>
       <c r="D358" s="5" t="n">
-        <v>10400000</v>
+        <v>50540</v>
       </c>
       <c r="E358" s="4" t="n">
-        <v>0.2007</v>
+        <v>0.0789</v>
       </c>
       <c r="F358" s="3" t="n">
-        <v>55.33</v>
+        <v>39.64</v>
       </c>
       <c r="G358" s="2" t="inlineStr"/>
       <c r="H358" s="3" t="n">
         <v>2.12</v>
       </c>
-      <c r="I358" s="2" t="inlineStr"/>
+      <c r="I358" s="4" t="n">
+        <v>-0.08929999999999999</v>
+      </c>
       <c r="J358" s="4" t="n">
-        <v>-0.8944</v>
+        <v>0.4032</v>
       </c>
       <c r="K358" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L358" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST BURSA</t>
         </is>
       </c>
       <c r="M358" s="2" t="inlineStr"/>
@@ -16071,42 +16073,42 @@
     <row r="359">
       <c r="A359" s="6" t="inlineStr">
         <is>
-          <t>SONME</t>
-        </is>
-      </c>
-      <c r="B359" s="7" t="n">
-        <v>134.3</v>
+          <t>EGEEN</t>
+        </is>
+      </c>
+      <c r="B359" s="9" t="n">
+        <v>5830</v>
       </c>
       <c r="C359" s="8" t="n">
-        <v>-0.0118</v>
+        <v>-0.0239</v>
       </c>
       <c r="D359" s="9" t="n">
-        <v>50540</v>
+        <v>17130</v>
       </c>
       <c r="E359" s="8" t="n">
-        <v>0.0789</v>
+        <v>0.3637</v>
       </c>
       <c r="F359" s="7" t="n">
-        <v>39.64</v>
+        <v>38.68</v>
       </c>
       <c r="G359" s="6" t="inlineStr"/>
       <c r="H359" s="7" t="n">
-        <v>2.12</v>
+        <v>2.17</v>
       </c>
       <c r="I359" s="8" t="n">
-        <v>-0.08929999999999999</v>
+        <v>-0.0341</v>
       </c>
       <c r="J359" s="8" t="n">
-        <v>0.4032</v>
+        <v>0.3126</v>
       </c>
       <c r="K359" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L359" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST BURSA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST YILDIZ, BIST İZMİR</t>
         </is>
       </c>
       <c r="M359" s="6" t="inlineStr"/>
@@ -16114,42 +16116,42 @@
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>EGEEN</t>
-        </is>
-      </c>
-      <c r="B360" s="5" t="n">
-        <v>5830</v>
+          <t>RUZYE</t>
+        </is>
+      </c>
+      <c r="B360" s="3" t="n">
+        <v>11.94</v>
       </c>
       <c r="C360" s="4" t="n">
-        <v>-0.0239</v>
+        <v>-0.0348</v>
       </c>
       <c r="D360" s="5" t="n">
-        <v>17130</v>
+        <v>8570000</v>
       </c>
       <c r="E360" s="4" t="n">
-        <v>0.3637</v>
+        <v>0.6456000000000001</v>
       </c>
       <c r="F360" s="3" t="n">
-        <v>38.68</v>
+        <v>38.71</v>
       </c>
       <c r="G360" s="2" t="inlineStr"/>
       <c r="H360" s="3" t="n">
-        <v>2.17</v>
+        <v>2.19</v>
       </c>
       <c r="I360" s="4" t="n">
-        <v>-0.0341</v>
+        <v>-0.0029</v>
       </c>
       <c r="J360" s="4" t="n">
-        <v>0.3126</v>
+        <v>-3.8066</v>
       </c>
       <c r="K360" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L360" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST YILDIZ, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST ANA, BIST KOBİ SANAYİ, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M360" s="2" t="inlineStr"/>
@@ -16157,42 +16159,40 @@
     <row r="361">
       <c r="A361" s="6" t="inlineStr">
         <is>
-          <t>RUZYE</t>
+          <t>SEYKM</t>
         </is>
       </c>
       <c r="B361" s="7" t="n">
-        <v>11.94</v>
+        <v>5.43</v>
       </c>
       <c r="C361" s="8" t="n">
-        <v>-0.0348</v>
+        <v>-0.0018</v>
       </c>
       <c r="D361" s="9" t="n">
-        <v>8570000</v>
-      </c>
-      <c r="E361" s="8" t="n">
-        <v>0.6456000000000001</v>
-      </c>
+        <v>4310000</v>
+      </c>
+      <c r="E361" s="6" t="inlineStr"/>
       <c r="F361" s="7" t="n">
-        <v>38.71</v>
+        <v>56.78</v>
       </c>
       <c r="G361" s="6" t="inlineStr"/>
       <c r="H361" s="7" t="n">
         <v>2.19</v>
       </c>
       <c r="I361" s="8" t="n">
-        <v>-0.0029</v>
+        <v>-0.0332</v>
       </c>
       <c r="J361" s="8" t="n">
-        <v>-3.8066</v>
+        <v>-0.8992</v>
       </c>
       <c r="K361" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Sağlık teknolojisi</t>
         </is>
       </c>
       <c r="L361" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST ANA, BIST KOBİ SANAYİ, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KOBİ SANAYİ, BIST MANİSA</t>
         </is>
       </c>
       <c r="M361" s="6" t="inlineStr"/>
@@ -16200,40 +16200,44 @@
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>SEYKM</t>
+          <t>SEGMN</t>
         </is>
       </c>
       <c r="B362" s="3" t="n">
-        <v>5.43</v>
+        <v>61.75</v>
       </c>
       <c r="C362" s="4" t="n">
-        <v>-0.0018</v>
+        <v>-0.0672</v>
       </c>
       <c r="D362" s="5" t="n">
-        <v>4310000</v>
-      </c>
-      <c r="E362" s="2" t="inlineStr"/>
+        <v>5080000</v>
+      </c>
+      <c r="E362" s="4" t="n">
+        <v>0.2515</v>
+      </c>
       <c r="F362" s="3" t="n">
-        <v>56.78</v>
-      </c>
-      <c r="G362" s="2" t="inlineStr"/>
+        <v>51.67</v>
+      </c>
+      <c r="G362" s="3" t="n">
+        <v>40.32</v>
+      </c>
       <c r="H362" s="3" t="n">
-        <v>2.19</v>
+        <v>2.2</v>
       </c>
       <c r="I362" s="4" t="n">
-        <v>-0.0332</v>
+        <v>0.0669</v>
       </c>
       <c r="J362" s="4" t="n">
-        <v>-0.8992</v>
+        <v>4.7457</v>
       </c>
       <c r="K362" s="2" t="inlineStr">
         <is>
-          <t>Sağlık teknolojisi</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L362" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KOBİ SANAYİ, BIST MANİSA</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ANA, BIST ANKARA</t>
         </is>
       </c>
       <c r="M362" s="2" t="inlineStr"/>
@@ -16241,44 +16245,44 @@
     <row r="363">
       <c r="A363" s="6" t="inlineStr">
         <is>
-          <t>SEGMN</t>
+          <t>MPARK</t>
         </is>
       </c>
       <c r="B363" s="7" t="n">
-        <v>61.75</v>
+        <v>462</v>
       </c>
       <c r="C363" s="8" t="n">
-        <v>-0.0672</v>
+        <v>-0.0479</v>
       </c>
       <c r="D363" s="9" t="n">
-        <v>5080000</v>
+        <v>966010</v>
       </c>
       <c r="E363" s="8" t="n">
-        <v>0.2515</v>
+        <v>0.4234000000000001</v>
       </c>
       <c r="F363" s="7" t="n">
-        <v>51.67</v>
+        <v>49.61</v>
       </c>
       <c r="G363" s="7" t="n">
-        <v>40.32</v>
+        <v>15.23</v>
       </c>
       <c r="H363" s="7" t="n">
-        <v>2.2</v>
+        <v>2.21</v>
       </c>
       <c r="I363" s="8" t="n">
-        <v>0.0669</v>
+        <v>0.1752</v>
       </c>
       <c r="J363" s="8" t="n">
-        <v>4.7457</v>
+        <v>0.1408</v>
       </c>
       <c r="K363" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Sağlık hizmetleri</t>
         </is>
       </c>
       <c r="L363" s="6" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ANA, BIST ANKARA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST SÜRDÜRÜLEBİLİRLİK, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK, STOXX Emerging Markets 1500</t>
         </is>
       </c>
       <c r="M363" s="6" t="inlineStr"/>
@@ -16286,44 +16290,40 @@
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>MPARK</t>
+          <t>KNFRT</t>
         </is>
       </c>
       <c r="B364" s="3" t="n">
-        <v>462</v>
+        <v>12.26</v>
       </c>
       <c r="C364" s="4" t="n">
-        <v>-0.0479</v>
+        <v>-0.0033</v>
       </c>
       <c r="D364" s="5" t="n">
-        <v>966010</v>
+        <v>4790000</v>
       </c>
       <c r="E364" s="4" t="n">
-        <v>0.4234000000000001</v>
+        <v>0.2239</v>
       </c>
       <c r="F364" s="3" t="n">
-        <v>49.61</v>
-      </c>
-      <c r="G364" s="3" t="n">
-        <v>15.23</v>
-      </c>
+        <v>52.14</v>
+      </c>
+      <c r="G364" s="2" t="inlineStr"/>
       <c r="H364" s="3" t="n">
-        <v>2.21</v>
+        <v>2.22</v>
       </c>
       <c r="I364" s="4" t="n">
-        <v>0.1752</v>
-      </c>
-      <c r="J364" s="4" t="n">
-        <v>0.1408</v>
-      </c>
+        <v>-0.09710000000000001</v>
+      </c>
+      <c r="J364" s="2" t="inlineStr"/>
       <c r="K364" s="2" t="inlineStr">
         <is>
-          <t>Sağlık hizmetleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L364" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST SÜRDÜRÜLEBİLİRLİK, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK, STOXX Emerging Markets 1500</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M364" s="2" t="inlineStr"/>
@@ -16331,40 +16331,40 @@
     <row r="365">
       <c r="A365" s="6" t="inlineStr">
         <is>
-          <t>KNFRT</t>
+          <t>MEKAG</t>
         </is>
       </c>
       <c r="B365" s="7" t="n">
-        <v>12.26</v>
+        <v>3.97</v>
       </c>
       <c r="C365" s="8" t="n">
-        <v>-0.0033</v>
+        <v>-0.0173</v>
       </c>
       <c r="D365" s="9" t="n">
-        <v>4790000</v>
+        <v>29960000</v>
       </c>
       <c r="E365" s="8" t="n">
-        <v>0.2239</v>
+        <v>0.2704</v>
       </c>
       <c r="F365" s="7" t="n">
-        <v>52.14</v>
+        <v>31.27</v>
       </c>
       <c r="G365" s="6" t="inlineStr"/>
       <c r="H365" s="7" t="n">
-        <v>2.22</v>
+        <v>2.24</v>
       </c>
       <c r="I365" s="8" t="n">
-        <v>-0.09710000000000001</v>
+        <v>-0.0452</v>
       </c>
       <c r="J365" s="6" t="inlineStr"/>
       <c r="K365" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L365" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM TÜM, BIST ANA, BIST ANKARA</t>
         </is>
       </c>
       <c r="M365" s="6" t="inlineStr"/>
@@ -16372,30 +16372,32 @@
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>MEKAG</t>
+          <t>SARKY</t>
         </is>
       </c>
       <c r="B366" s="3" t="n">
-        <v>3.97</v>
+        <v>29</v>
       </c>
       <c r="C366" s="4" t="n">
-        <v>-0.0173</v>
+        <v>-0.08169999999999999</v>
       </c>
       <c r="D366" s="5" t="n">
-        <v>29960000</v>
+        <v>20860000</v>
       </c>
       <c r="E366" s="4" t="n">
-        <v>0.2704</v>
+        <v>0.6767</v>
       </c>
       <c r="F366" s="3" t="n">
-        <v>31.27</v>
-      </c>
-      <c r="G366" s="2" t="inlineStr"/>
+        <v>50.24</v>
+      </c>
+      <c r="G366" s="3" t="n">
+        <v>81.41</v>
+      </c>
       <c r="H366" s="3" t="n">
-        <v>2.24</v>
+        <v>2.25</v>
       </c>
       <c r="I366" s="4" t="n">
-        <v>-0.0452</v>
+        <v>0.0343</v>
       </c>
       <c r="J366" s="2" t="inlineStr"/>
       <c r="K366" s="2" t="inlineStr">
@@ -16405,7 +16407,7 @@
       </c>
       <c r="L366" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM TÜM, BIST ANA, BIST ANKARA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU, BIST KATILIM 50, BIST KATILIM TEMETTU, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M366" s="2" t="inlineStr"/>
@@ -16413,42 +16415,42 @@
     <row r="367">
       <c r="A367" s="6" t="inlineStr">
         <is>
-          <t>SARKY</t>
+          <t>ERSU</t>
         </is>
       </c>
       <c r="B367" s="7" t="n">
-        <v>29</v>
+        <v>26.64</v>
       </c>
       <c r="C367" s="8" t="n">
-        <v>-0.08169999999999999</v>
+        <v>-0.0133</v>
       </c>
       <c r="D367" s="9" t="n">
-        <v>20860000</v>
+        <v>700990</v>
       </c>
       <c r="E367" s="8" t="n">
-        <v>0.6767</v>
+        <v>0.7902</v>
       </c>
       <c r="F367" s="7" t="n">
-        <v>50.24</v>
-      </c>
-      <c r="G367" s="7" t="n">
-        <v>81.41</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="G367" s="6" t="inlineStr"/>
       <c r="H367" s="7" t="n">
         <v>2.25</v>
       </c>
       <c r="I367" s="8" t="n">
-        <v>0.0343</v>
-      </c>
-      <c r="J367" s="6" t="inlineStr"/>
+        <v>-0.2756</v>
+      </c>
+      <c r="J367" s="8" t="n">
+        <v>0.5871999999999999</v>
+      </c>
       <c r="K367" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L367" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU, BIST KATILIM 50, BIST KATILIM TEMETTU, BIST KOCAELI</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KOBİ SANAYİ, BIST KONYA</t>
         </is>
       </c>
       <c r="M367" s="6" t="inlineStr"/>
@@ -16456,33 +16458,33 @@
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>ERSU</t>
+          <t>OBAMS</t>
         </is>
       </c>
       <c r="B368" s="3" t="n">
-        <v>26.64</v>
+        <v>8.59</v>
       </c>
       <c r="C368" s="4" t="n">
-        <v>-0.0133</v>
+        <v>-0.0035</v>
       </c>
       <c r="D368" s="5" t="n">
-        <v>700990</v>
+        <v>83560000</v>
       </c>
       <c r="E368" s="4" t="n">
-        <v>0.7902</v>
+        <v>0.2611</v>
       </c>
       <c r="F368" s="3" t="n">
-        <v>53</v>
+        <v>56.69</v>
       </c>
       <c r="G368" s="2" t="inlineStr"/>
       <c r="H368" s="3" t="n">
         <v>2.25</v>
       </c>
       <c r="I368" s="4" t="n">
-        <v>-0.2756</v>
+        <v>-0.1977</v>
       </c>
       <c r="J368" s="4" t="n">
-        <v>0.5871999999999999</v>
+        <v>-0.0043</v>
       </c>
       <c r="K368" s="2" t="inlineStr">
         <is>
@@ -16491,7 +16493,7 @@
       </c>
       <c r="L368" s="2" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KOBİ SANAYİ, BIST KONYA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M368" s="2" t="inlineStr"/>
@@ -16499,42 +16501,44 @@
     <row r="369">
       <c r="A369" s="6" t="inlineStr">
         <is>
-          <t>OBAMS</t>
+          <t>KLKIM</t>
         </is>
       </c>
       <c r="B369" s="7" t="n">
-        <v>8.59</v>
+        <v>32.04</v>
       </c>
       <c r="C369" s="8" t="n">
-        <v>-0.0035</v>
+        <v>-0.0172</v>
       </c>
       <c r="D369" s="9" t="n">
-        <v>83560000</v>
+        <v>3580000</v>
       </c>
       <c r="E369" s="8" t="n">
-        <v>0.2611</v>
+        <v>0.2637</v>
       </c>
       <c r="F369" s="7" t="n">
-        <v>56.69</v>
-      </c>
-      <c r="G369" s="6" t="inlineStr"/>
+        <v>36.02</v>
+      </c>
+      <c r="G369" s="7" t="n">
+        <v>13.49</v>
+      </c>
       <c r="H369" s="7" t="n">
-        <v>2.25</v>
+        <v>2.27</v>
       </c>
       <c r="I369" s="8" t="n">
-        <v>-0.1977</v>
+        <v>0.2016</v>
       </c>
       <c r="J369" s="8" t="n">
-        <v>-0.0043</v>
+        <v>0.5552</v>
       </c>
       <c r="K369" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L369" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST İSTANBUL, BIST YILDIZ, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M369" s="6" t="inlineStr"/>
@@ -16542,44 +16546,42 @@
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>KLKIM</t>
+          <t>HURGZ</t>
         </is>
       </c>
       <c r="B370" s="3" t="n">
-        <v>32.04</v>
+        <v>8.77</v>
       </c>
       <c r="C370" s="4" t="n">
-        <v>-0.0172</v>
+        <v>-0.0201</v>
       </c>
       <c r="D370" s="5" t="n">
-        <v>3580000</v>
+        <v>27210000</v>
       </c>
       <c r="E370" s="4" t="n">
-        <v>0.2637</v>
+        <v>0.1879</v>
       </c>
       <c r="F370" s="3" t="n">
-        <v>36.02</v>
-      </c>
-      <c r="G370" s="3" t="n">
-        <v>13.49</v>
-      </c>
+        <v>62.4</v>
+      </c>
+      <c r="G370" s="2" t="inlineStr"/>
       <c r="H370" s="3" t="n">
         <v>2.27</v>
       </c>
       <c r="I370" s="4" t="n">
-        <v>0.2016</v>
+        <v>-0.4406</v>
       </c>
       <c r="J370" s="4" t="n">
-        <v>0.5552</v>
+        <v>-11.3341</v>
       </c>
       <c r="K370" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L370" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST İSTANBUL, BIST YILDIZ, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M370" s="2" t="inlineStr"/>
@@ -25909,21 +25911,23 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>2.73</v>
+        <v>6.44</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0</v>
+        <v>0.0733</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>142720000</v>
-      </c>
-      <c r="E587" s="6" t="inlineStr"/>
+        <v>19120000</v>
+      </c>
+      <c r="E587" s="8" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F587" s="7" t="n">
-        <v>45.93</v>
+        <v>70.31</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25936,7 +25940,7 @@
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25944,34 +25948,40 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>13.96</v>
+        <v>5.97</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0285</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>30370000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>35800000</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>49.07</v>
+        <v>49.23</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="I588" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J588" s="4" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25979,23 +25989,21 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>6.44</v>
+        <v>36.4</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0733</v>
+        <v>0.0196</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>19120000</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>6480000</v>
+      </c>
+      <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>70.31</v>
+        <v>58.24</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26003,12 +26011,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26016,40 +26024,40 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>2.48</v>
+        <v>142.7</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.008</v>
+        <v>0.061</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>21880000</v>
+        <v>995180</v>
       </c>
       <c r="E590" s="4" t="n">
-        <v>1</v>
+        <v>0.1071</v>
       </c>
       <c r="F590" s="3" t="n">
-        <v>35.12</v>
+        <v>48.18</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="4" t="n">
-        <v>-191.6342</v>
+        <v>-3.6635</v>
       </c>
       <c r="J590" s="4" t="n">
-        <v>-0.8093</v>
+        <v>-0.4897</v>
       </c>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26057,21 +26065,21 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>198.4</v>
+        <v>18.16</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0345</v>
+        <v>0.0145</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>8520000</v>
+        <v>45490000</v>
       </c>
       <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>61.52</v>
+        <v>52.57</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26084,7 +26092,7 @@
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26092,38 +26100,34 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>26.02</v>
+        <v>178.6</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.008399999999999999</v>
+        <v>-0.0341</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>883760</v>
-      </c>
-      <c r="E592" s="4" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>8620000</v>
+      </c>
+      <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>43.34</v>
+        <v>38.77</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
       <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="4" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26131,21 +26135,21 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>42.32</v>
+        <v>73.8</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.0272</v>
+        <v>-0.0238</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>5980000</v>
+        <v>174630</v>
       </c>
       <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>53.18</v>
+        <v>10.48</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
@@ -26153,34 +26157,32 @@
       <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr"/>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>17.05</v>
+        <v>240.1</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0512</v>
+        <v>-0.02</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>48680000</v>
-      </c>
-      <c r="E594" s="2" t="inlineStr"/>
+        <v>10620</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F594" s="3" t="n">
-        <v>49.01</v>
+        <v>43.77</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26188,53 +26190,43 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr"/>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>142.7</v>
+        <v>17.05</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.061</v>
+        <v>-0.0512</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>995180</v>
-      </c>
-      <c r="E595" s="8" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>48680000</v>
+      </c>
+      <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>48.18</v>
+        <v>49.01</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J595" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I595" s="6" t="inlineStr"/>
+      <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26242,23 +26234,21 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>30.64</v>
+        <v>18.53</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.07820000000000001</v>
+        <v>0.0011</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>16140000</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>55440000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>52.53</v>
+        <v>35.89</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26266,12 +26256,12 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26279,34 +26269,42 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>18.53</v>
+        <v>34.68</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0011</v>
+        <v>-0.0181</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>55440000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>5190000</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.3528</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>35.89</v>
-      </c>
-      <c r="G597" s="6" t="inlineStr"/>
+        <v>43.26</v>
+      </c>
+      <c r="G597" s="7" t="n">
+        <v>13.71</v>
+      </c>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26314,38 +26312,38 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>65.15000000000001</v>
+        <v>26.02</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0585</v>
+        <v>-0.008399999999999999</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>869750</v>
+        <v>883760</v>
       </c>
       <c r="E598" s="4" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.9698</v>
       </c>
       <c r="F598" s="3" t="n">
-        <v>49.58</v>
+        <v>43.34</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
       <c r="J598" s="4" t="n">
-        <v>0.1431</v>
+        <v>0.6453</v>
       </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26353,21 +26351,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>77.25</v>
+        <v>13.96</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.09960000000000001</v>
+        <v>-0.0285</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>29900000</v>
+        <v>30370000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>88.89</v>
+        <v>49.07</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26375,12 +26373,12 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26388,21 +26386,21 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>36.4</v>
+        <v>2.73</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0196</v>
+        <v>0</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>6480000</v>
+        <v>142720000</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>58.24</v>
+        <v>45.93</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26410,12 +26408,12 @@
       <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26423,56 +26421,48 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>28.4</v>
+        <v>78.62</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0373</v>
+        <v>-0.0067</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>23640000</v>
+        <v>11350000</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>55.6</v>
+        <v>37.39</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="6" t="inlineStr"/>
       <c r="J601" s="6" t="inlineStr"/>
-      <c r="K601" s="6" t="inlineStr">
-        <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+      <c r="K601" s="6" t="inlineStr"/>
+      <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>18.16</v>
+        <v>77.25</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0145</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>45490000</v>
+        <v>29900000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>52.57</v>
+        <v>88.89</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26480,12 +26470,12 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26493,35 +26483,35 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>9.93</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0793</v>
+        <v>0.0162</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>757940</v>
+        <v>48030</v>
       </c>
       <c r="E603" s="8" t="n">
-        <v>0.95</v>
+        <v>0.58</v>
       </c>
       <c r="F603" s="7" t="n">
-        <v>61.27</v>
+        <v>36.59</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
       <c r="I603" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-9.409700000000001</v>
       </c>
       <c r="J603" s="8" t="n">
-        <v>-0.4678</v>
+        <v>-4.155</v>
       </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Taşımacılık</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr"/>
@@ -26530,50 +26520,56 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>78.62</v>
+        <v>28.4</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0067</v>
+        <v>-0.0373</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>11350000</v>
+        <v>23640000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>37.39</v>
+        <v>55.6</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
       <c r="I604" s="2" t="inlineStr"/>
       <c r="J604" s="2" t="inlineStr"/>
-      <c r="K604" s="2" t="inlineStr"/>
-      <c r="L604" s="2" t="inlineStr"/>
+      <c r="K604" s="2" t="inlineStr">
+        <is>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr">
+        <is>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>240.1</v>
+        <v>6.06</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.02</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>10620</v>
-      </c>
-      <c r="E605" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>7340000</v>
+      </c>
+      <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>43.77</v>
+        <v>45.24</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26581,7 +26577,7 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr"/>
@@ -26590,34 +26586,40 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>178.6</v>
+        <v>2.48</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0341</v>
+        <v>-0.008</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>8620000</v>
-      </c>
-      <c r="E606" s="2" t="inlineStr"/>
+        <v>21880000</v>
+      </c>
+      <c r="E606" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="F606" s="3" t="n">
-        <v>38.77</v>
+        <v>35.12</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="2" t="inlineStr"/>
-      <c r="J606" s="2" t="inlineStr"/>
+      <c r="I606" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J606" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26625,40 +26627,36 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>5.97</v>
+        <v>30.64</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.09939999999999999</v>
+        <v>-0.07820000000000001</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>35800000</v>
+        <v>16140000</v>
       </c>
       <c r="E607" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.2667</v>
       </c>
       <c r="F607" s="7" t="n">
-        <v>49.23</v>
+        <v>52.53</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J607" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I607" s="6" t="inlineStr"/>
+      <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26666,29 +26664,35 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>6.06</v>
+        <v>9.93</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>-0.008199999999999999</v>
+        <v>0.0793</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>7340000</v>
-      </c>
-      <c r="E608" s="2" t="inlineStr"/>
+        <v>757940</v>
+      </c>
+      <c r="E608" s="4" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F608" s="3" t="n">
-        <v>45.24</v>
+        <v>61.27</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
-      <c r="I608" s="2" t="inlineStr"/>
-      <c r="J608" s="2" t="inlineStr"/>
+      <c r="I608" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J608" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr"/>
@@ -26697,21 +26701,21 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>73.8</v>
+        <v>42.32</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>-0.0238</v>
+        <v>0.0272</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>174630</v>
+        <v>5980000</v>
       </c>
       <c r="E609" s="6" t="inlineStr"/>
       <c r="F609" s="7" t="n">
-        <v>10.48</v>
+        <v>53.18</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
@@ -26719,51 +26723,47 @@
       <c r="J609" s="6" t="inlineStr"/>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L609" s="6" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L609" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M609" s="6" t="inlineStr"/>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>34.68</v>
+        <v>198.4</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.0181</v>
+        <v>-0.0345</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>5190000</v>
-      </c>
-      <c r="E610" s="4" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>8520000</v>
+      </c>
+      <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>43.26</v>
-      </c>
-      <c r="G610" s="3" t="n">
-        <v>13.71</v>
-      </c>
+        <v>61.52</v>
+      </c>
+      <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
-      <c r="I610" s="4" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J610" s="4" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I610" s="2" t="inlineStr"/>
+      <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M610" s="2" t="inlineStr"/>
@@ -26771,38 +26771,40 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>69.09999999999999</v>
+        <v>65.15000000000001</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>0.0162</v>
+        <v>-0.0585</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>48030</v>
+        <v>869750</v>
       </c>
       <c r="E611" s="8" t="n">
-        <v>0.58</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F611" s="7" t="n">
-        <v>36.59</v>
+        <v>49.58</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
+      <c r="I611" s="6" t="inlineStr"/>
       <c r="J611" s="8" t="n">
-        <v>-4.155</v>
+        <v>0.1431</v>
       </c>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L611" s="6" t="inlineStr"/>
+          <t>Teknoloji hizmetleri</t>
+        </is>
+      </c>
+      <c r="L611" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M611" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26827,7 +26829,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>19.05.2026 09:30</t>
+          <t>19.05.2026 10:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 19.05.2026 11:30 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-19.xlsx
+++ b/data/bist_screener_2026-05-19.xlsx
@@ -25911,23 +25911,21 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>6.44</v>
+        <v>36.4</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0733</v>
+        <v>0.0196</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>19120000</v>
-      </c>
-      <c r="E587" s="8" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>6480000</v>
+      </c>
+      <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>70.31</v>
+        <v>58.24</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25935,12 +25933,12 @@
       <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25948,32 +25946,28 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>5.97</v>
+        <v>6.44</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.09939999999999999</v>
+        <v>0.0733</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>35800000</v>
+        <v>19120000</v>
       </c>
       <c r="E588" s="4" t="n">
-        <v>0.1672</v>
+        <v>0.8667</v>
       </c>
       <c r="F588" s="3" t="n">
-        <v>49.23</v>
+        <v>70.31</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J588" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I588" s="2" t="inlineStr"/>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -25981,7 +25975,7 @@
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25989,21 +25983,21 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>36.4</v>
+        <v>178.6</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0196</v>
+        <v>-0.0341</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>6480000</v>
+        <v>8620000</v>
       </c>
       <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>58.24</v>
+        <v>38.77</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26011,12 +26005,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26024,40 +26018,34 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>142.7</v>
+        <v>13.96</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.061</v>
+        <v>-0.0285</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>995180</v>
-      </c>
-      <c r="E590" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>30370000</v>
+      </c>
+      <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>48.18</v>
+        <v>49.07</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J590" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I590" s="2" t="inlineStr"/>
+      <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26065,124 +26053,140 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>18.16</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0145</v>
+        <v>0.0162</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>45490000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>48030</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>52.57</v>
+        <v>36.59</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="6" t="inlineStr"/>
+      <c r="I591" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J591" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr"/>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>178.6</v>
+        <v>9.93</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0341</v>
+        <v>0.0793</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>8620000</v>
-      </c>
-      <c r="E592" s="2" t="inlineStr"/>
+        <v>757940</v>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F592" s="3" t="n">
-        <v>38.77</v>
+        <v>61.27</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="2" t="inlineStr"/>
+      <c r="I592" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J592" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr"/>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>73.8</v>
+        <v>34.68</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0238</v>
+        <v>-0.0181</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>174630</v>
-      </c>
-      <c r="E593" s="6" t="inlineStr"/>
+        <v>5190000</v>
+      </c>
+      <c r="E593" s="8" t="n">
+        <v>0.3528</v>
+      </c>
       <c r="F593" s="7" t="n">
-        <v>10.48</v>
-      </c>
-      <c r="G593" s="6" t="inlineStr"/>
+        <v>43.26</v>
+      </c>
+      <c r="G593" s="7" t="n">
+        <v>13.71</v>
+      </c>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="6" t="inlineStr"/>
+      <c r="I593" s="8" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J593" s="8" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr"/>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>240.1</v>
+        <v>30.64</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.02</v>
+        <v>-0.07820000000000001</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>10620</v>
+        <v>16140000</v>
       </c>
       <c r="E594" s="4" t="n">
-        <v>0.2578</v>
+        <v>0.2667</v>
       </c>
       <c r="F594" s="3" t="n">
-        <v>43.77</v>
+        <v>52.53</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26190,43 +26194,51 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>17.05</v>
+        <v>65.15000000000001</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0512</v>
+        <v>-0.0585</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>48680000</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
+        <v>869750</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F595" s="7" t="n">
-        <v>49.01</v>
+        <v>49.58</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="6" t="inlineStr"/>
+      <c r="J595" s="8" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26234,34 +26246,40 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>18.53</v>
+        <v>2.48</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0011</v>
+        <v>-0.008</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>55440000</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>21880000</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>35.89</v>
+        <v>35.12</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J596" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26269,81 +26287,65 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>34.68</v>
+        <v>6.06</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0181</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>5190000</v>
-      </c>
-      <c r="E597" s="8" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>7340000</v>
+      </c>
+      <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>43.26</v>
-      </c>
-      <c r="G597" s="7" t="n">
-        <v>13.71</v>
-      </c>
+        <v>45.24</v>
+      </c>
+      <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="8" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J597" s="8" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I597" s="6" t="inlineStr"/>
+      <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>26.02</v>
+        <v>18.53</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.008399999999999999</v>
+        <v>0.0011</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>883760</v>
-      </c>
-      <c r="E598" s="4" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>55440000</v>
+      </c>
+      <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>43.34</v>
+        <v>35.89</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="4" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26351,36 +26353,28 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>13.96</v>
+        <v>78.62</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0285</v>
+        <v>-0.0067</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>30370000</v>
+        <v>11350000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>49.07</v>
+        <v>37.39</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
       <c r="I599" s="6" t="inlineStr"/>
       <c r="J599" s="6" t="inlineStr"/>
-      <c r="K599" s="6" t="inlineStr">
-        <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+      <c r="K599" s="6" t="inlineStr"/>
+      <c r="L599" s="6" t="inlineStr"/>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
@@ -26421,48 +26415,52 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>78.62</v>
+        <v>73.8</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0067</v>
+        <v>-0.0238</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>11350000</v>
+        <v>174630</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>37.39</v>
+        <v>10.48</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="6" t="inlineStr"/>
       <c r="J601" s="6" t="inlineStr"/>
-      <c r="K601" s="6" t="inlineStr"/>
+      <c r="K601" s="6" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
       <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>77.25</v>
+        <v>17.05</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.09960000000000001</v>
+        <v>-0.0512</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>29900000</v>
+        <v>48680000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>88.89</v>
+        <v>49.01</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26470,12 +26468,12 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26483,71 +26481,75 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>69.09999999999999</v>
+        <v>42.32</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0162</v>
+        <v>0.0272</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>48030</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.58</v>
-      </c>
+        <v>5980000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>36.59</v>
+        <v>53.18</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>28.4</v>
+        <v>5.97</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0373</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>23640000</v>
-      </c>
-      <c r="E604" s="2" t="inlineStr"/>
+        <v>35800000</v>
+      </c>
+      <c r="E604" s="4" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F604" s="3" t="n">
-        <v>55.6</v>
+        <v>49.23</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="2" t="inlineStr"/>
-      <c r="J604" s="2" t="inlineStr"/>
+      <c r="I604" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J604" s="4" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26555,21 +26557,21 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>6.06</v>
+        <v>18.16</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.008199999999999999</v>
+        <v>0.0145</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>7340000</v>
+        <v>45490000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>45.24</v>
+        <v>52.57</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26577,49 +26579,51 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L605" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>2.48</v>
+        <v>26.02</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.008</v>
+        <v>-0.008399999999999999</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>21880000</v>
+        <v>883760</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>1</v>
+        <v>0.9698</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>35.12</v>
+        <v>43.34</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
+      <c r="I606" s="2" t="inlineStr"/>
       <c r="J606" s="4" t="n">
-        <v>-0.8093</v>
+        <v>0.6453</v>
       </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26627,23 +26631,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>30.64</v>
+        <v>28.4</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.07820000000000001</v>
+        <v>-0.0373</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>16140000</v>
-      </c>
-      <c r="E607" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>23640000</v>
+      </c>
+      <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>52.53</v>
+        <v>55.6</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26651,12 +26653,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26664,58 +26666,58 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>9.93</v>
+        <v>198.4</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0793</v>
+        <v>-0.0345</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>757940</v>
-      </c>
-      <c r="E608" s="4" t="n">
-        <v>0.95</v>
-      </c>
+        <v>8520000</v>
+      </c>
+      <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>61.27</v>
+        <v>61.52</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
-      <c r="I608" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J608" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I608" s="2" t="inlineStr"/>
+      <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L608" s="2" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L608" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M608" s="2" t="inlineStr"/>
     </row>
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>42.32</v>
+        <v>240.1</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.0272</v>
+        <v>-0.02</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>5980000</v>
-      </c>
-      <c r="E609" s="6" t="inlineStr"/>
+        <v>10620</v>
+      </c>
+      <c r="E609" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F609" s="7" t="n">
-        <v>53.18</v>
+        <v>43.77</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
@@ -26723,34 +26725,30 @@
       <c r="J609" s="6" t="inlineStr"/>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L609" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L609" s="6" t="inlineStr"/>
       <c r="M609" s="6" t="inlineStr"/>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>198.4</v>
+        <v>77.25</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.0345</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>8520000</v>
+        <v>29900000</v>
       </c>
       <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>61.52</v>
+        <v>88.89</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
@@ -26758,7 +26756,7 @@
       <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr">
@@ -26771,38 +26769,40 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>65.15000000000001</v>
+        <v>142.7</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.0585</v>
+        <v>0.061</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>869750</v>
+        <v>995180</v>
       </c>
       <c r="E611" s="8" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.1071</v>
       </c>
       <c r="F611" s="7" t="n">
-        <v>49.58</v>
+        <v>48.18</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="6" t="inlineStr"/>
+      <c r="I611" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
       <c r="J611" s="8" t="n">
-        <v>0.1431</v>
+        <v>-0.4897</v>
       </c>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26829,7 +26829,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>19.05.2026 10:30</t>
+          <t>19.05.2026 11:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 19.05.2026 12:30 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-19.xlsx
+++ b/data/bist_screener_2026-05-19.xlsx
@@ -25911,21 +25911,21 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>36.4</v>
+        <v>13.96</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0196</v>
+        <v>-0.0285</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>6480000</v>
+        <v>30370000</v>
       </c>
       <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>58.24</v>
+        <v>49.07</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25933,12 +25933,12 @@
       <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25946,23 +25946,21 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>6.44</v>
+        <v>18.16</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0733</v>
+        <v>0.0145</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>19120000</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>45490000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>70.31</v>
+        <v>52.57</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25970,12 +25968,12 @@
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25983,105 +25981,95 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>178.6</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0341</v>
+        <v>0.0162</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>8620000</v>
-      </c>
-      <c r="E589" s="6" t="inlineStr"/>
+        <v>48030</v>
+      </c>
+      <c r="E589" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F589" s="7" t="n">
-        <v>38.77</v>
+        <v>36.59</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="6" t="inlineStr"/>
-      <c r="J589" s="6" t="inlineStr"/>
+      <c r="I589" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J589" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr"/>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>13.96</v>
+        <v>78.62</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0285</v>
+        <v>-0.0067</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>30370000</v>
+        <v>11350000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>49.07</v>
+        <v>37.39</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="2" t="inlineStr"/>
       <c r="J590" s="2" t="inlineStr"/>
-      <c r="K590" s="2" t="inlineStr">
-        <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L590" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+      <c r="K590" s="2" t="inlineStr"/>
+      <c r="L590" s="2" t="inlineStr"/>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>69.09999999999999</v>
+        <v>240.1</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0162</v>
+        <v>-0.02</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>48030</v>
+        <v>10620</v>
       </c>
       <c r="E591" s="8" t="n">
-        <v>0.58</v>
+        <v>0.2578</v>
       </c>
       <c r="F591" s="7" t="n">
-        <v>36.59</v>
+        <v>43.77</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J591" s="8" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I591" s="6" t="inlineStr"/>
+      <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr"/>
@@ -26090,103 +26078,93 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>9.93</v>
+        <v>77.25</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0793</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>757940</v>
-      </c>
-      <c r="E592" s="4" t="n">
-        <v>0.95</v>
-      </c>
+        <v>29900000</v>
+      </c>
+      <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>61.27</v>
+        <v>88.89</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J592" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I592" s="2" t="inlineStr"/>
+      <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr"/>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>34.68</v>
+        <v>9.93</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0181</v>
+        <v>0.0793</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>5190000</v>
+        <v>757940</v>
       </c>
       <c r="E593" s="8" t="n">
-        <v>0.3528</v>
+        <v>0.95</v>
       </c>
       <c r="F593" s="7" t="n">
-        <v>43.26</v>
-      </c>
-      <c r="G593" s="7" t="n">
-        <v>13.71</v>
-      </c>
+        <v>61.27</v>
+      </c>
+      <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
       <c r="I593" s="8" t="n">
-        <v>0.1029</v>
+        <v>-23.6291</v>
       </c>
       <c r="J593" s="8" t="n">
-        <v>-1.4864</v>
+        <v>-0.4678</v>
       </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr"/>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>30.64</v>
+        <v>2.73</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.07820000000000001</v>
+        <v>0</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>16140000</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>142720000</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>52.53</v>
+        <v>45.93</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26194,12 +26172,12 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26207,38 +26185,40 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>65.15000000000001</v>
+        <v>2.48</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0585</v>
+        <v>-0.008</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>869750</v>
+        <v>21880000</v>
       </c>
       <c r="E595" s="8" t="n">
-        <v>0.3695000000000001</v>
+        <v>1</v>
       </c>
       <c r="F595" s="7" t="n">
-        <v>49.58</v>
+        <v>35.12</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="6" t="inlineStr"/>
+      <c r="I595" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
       <c r="J595" s="8" t="n">
-        <v>0.1431</v>
+        <v>-0.8093</v>
       </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26246,40 +26226,36 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>2.48</v>
+        <v>6.44</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.008</v>
+        <v>0.0733</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>21880000</v>
+        <v>19120000</v>
       </c>
       <c r="E596" s="4" t="n">
-        <v>1</v>
+        <v>0.8667</v>
       </c>
       <c r="F596" s="3" t="n">
-        <v>35.12</v>
+        <v>70.31</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J596" s="4" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I596" s="2" t="inlineStr"/>
+      <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26287,21 +26263,21 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>6.06</v>
+        <v>198.4</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.008199999999999999</v>
+        <v>-0.0345</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>7340000</v>
+        <v>8520000</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>45.24</v>
+        <v>61.52</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26309,30 +26285,34 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>18.53</v>
+        <v>42.32</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.0011</v>
+        <v>0.0272</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>55440000</v>
+        <v>5980000</v>
       </c>
       <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>35.89</v>
+        <v>53.18</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26340,12 +26320,12 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26353,48 +26333,60 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>78.62</v>
+        <v>65.15000000000001</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0067</v>
+        <v>-0.0585</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>11350000</v>
-      </c>
-      <c r="E599" s="6" t="inlineStr"/>
+        <v>869750</v>
+      </c>
+      <c r="E599" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F599" s="7" t="n">
-        <v>37.39</v>
+        <v>49.58</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
       <c r="I599" s="6" t="inlineStr"/>
-      <c r="J599" s="6" t="inlineStr"/>
-      <c r="K599" s="6" t="inlineStr"/>
-      <c r="L599" s="6" t="inlineStr"/>
+      <c r="J599" s="8" t="n">
+        <v>0.1431</v>
+      </c>
+      <c r="K599" s="6" t="inlineStr">
+        <is>
+          <t>Teknoloji hizmetleri</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>2.73</v>
+        <v>18.53</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0</v>
+        <v>0.0011</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>142720000</v>
+        <v>55440000</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>45.93</v>
+        <v>35.89</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26407,7 +26399,7 @@
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26415,65 +26407,81 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>73.8</v>
+        <v>5.97</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0238</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>174630</v>
-      </c>
-      <c r="E601" s="6" t="inlineStr"/>
+        <v>35800000</v>
+      </c>
+      <c r="E601" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F601" s="7" t="n">
-        <v>10.48</v>
+        <v>49.23</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="6" t="inlineStr"/>
-      <c r="J601" s="6" t="inlineStr"/>
+      <c r="I601" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J601" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
         </is>
       </c>
-      <c r="L601" s="6" t="inlineStr"/>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>17.05</v>
+        <v>142.7</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0512</v>
+        <v>0.061</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>48680000</v>
-      </c>
-      <c r="E602" s="2" t="inlineStr"/>
+        <v>995180</v>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F602" s="3" t="n">
-        <v>49.01</v>
+        <v>48.18</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="2" t="inlineStr"/>
-      <c r="J602" s="2" t="inlineStr"/>
+      <c r="I602" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J602" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26481,21 +26489,21 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>42.32</v>
+        <v>73.8</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0272</v>
+        <v>-0.0238</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>5980000</v>
+        <v>174630</v>
       </c>
       <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>53.18</v>
+        <v>10.48</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
@@ -26503,53 +26511,51 @@
       <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr"/>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>5.97</v>
+        <v>34.68</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.09939999999999999</v>
+        <v>-0.0181</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>35800000</v>
+        <v>5190000</v>
       </c>
       <c r="E604" s="4" t="n">
-        <v>0.1672</v>
+        <v>0.3528</v>
       </c>
       <c r="F604" s="3" t="n">
-        <v>49.23</v>
-      </c>
-      <c r="G604" s="2" t="inlineStr"/>
+        <v>43.26</v>
+      </c>
+      <c r="G604" s="3" t="n">
+        <v>13.71</v>
+      </c>
       <c r="H604" s="2" t="inlineStr"/>
       <c r="I604" s="4" t="n">
-        <v>-5.3262</v>
+        <v>0.1029</v>
       </c>
       <c r="J604" s="4" t="n">
-        <v>-4.2562</v>
+        <v>-1.4864</v>
       </c>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26557,21 +26563,23 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>18.16</v>
+        <v>30.64</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0145</v>
+        <v>-0.07820000000000001</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>45490000</v>
-      </c>
-      <c r="E605" s="6" t="inlineStr"/>
+        <v>16140000</v>
+      </c>
+      <c r="E605" s="8" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F605" s="7" t="n">
-        <v>52.57</v>
+        <v>52.53</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26579,12 +26587,12 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26592,60 +26600,52 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>26.02</v>
+        <v>6.06</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.008399999999999999</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>883760</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>7340000</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>43.34</v>
+        <v>45.24</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
       <c r="I606" s="2" t="inlineStr"/>
-      <c r="J606" s="4" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr"/>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>28.4</v>
+        <v>178.6</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0373</v>
+        <v>-0.0341</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>23640000</v>
+        <v>8620000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>55.6</v>
+        <v>38.77</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26653,12 +26653,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26666,21 +26666,21 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>198.4</v>
+        <v>36.4</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>-0.0345</v>
+        <v>0.0196</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>8520000</v>
+        <v>6480000</v>
       </c>
       <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>61.52</v>
+        <v>58.24</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
@@ -26688,12 +26688,12 @@
       <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26701,54 +26701,60 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>240.1</v>
+        <v>26.02</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>-0.02</v>
+        <v>-0.008399999999999999</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>10620</v>
+        <v>883760</v>
       </c>
       <c r="E609" s="8" t="n">
-        <v>0.2578</v>
+        <v>0.9698</v>
       </c>
       <c r="F609" s="7" t="n">
-        <v>43.77</v>
+        <v>43.34</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
       <c r="I609" s="6" t="inlineStr"/>
-      <c r="J609" s="6" t="inlineStr"/>
+      <c r="J609" s="8" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L609" s="6" t="inlineStr"/>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L609" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+        </is>
+      </c>
       <c r="M609" s="6" t="inlineStr"/>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>77.25</v>
+        <v>17.05</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>0.09960000000000001</v>
+        <v>-0.0512</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>29900000</v>
+        <v>48680000</v>
       </c>
       <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>88.89</v>
+        <v>49.01</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
@@ -26756,12 +26762,12 @@
       <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M610" s="2" t="inlineStr"/>
@@ -26769,40 +26775,34 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>142.7</v>
+        <v>28.4</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>0.061</v>
+        <v>-0.0373</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>995180</v>
-      </c>
-      <c r="E611" s="8" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>23640000</v>
+      </c>
+      <c r="E611" s="6" t="inlineStr"/>
       <c r="F611" s="7" t="n">
-        <v>48.18</v>
+        <v>55.6</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J611" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I611" s="6" t="inlineStr"/>
+      <c r="J611" s="6" t="inlineStr"/>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26829,7 +26829,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>19.05.2026 11:30</t>
+          <t>19.05.2026 12:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 19.05.2026 13:30 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-19.xlsx
+++ b/data/bist_screener_2026-05-19.xlsx
@@ -19670,42 +19670,44 @@
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>EMKEL</t>
+          <t>LOGO</t>
         </is>
       </c>
       <c r="B442" s="3" t="n">
-        <v>23.74</v>
+        <v>155</v>
       </c>
       <c r="C442" s="4" t="n">
-        <v>-0.0389</v>
+        <v>-0.0252</v>
       </c>
       <c r="D442" s="5" t="n">
-        <v>11660000</v>
+        <v>1190000</v>
       </c>
       <c r="E442" s="4" t="n">
-        <v>0.9773999999999999</v>
+        <v>0.6459999999999999</v>
       </c>
       <c r="F442" s="3" t="n">
-        <v>46.43</v>
-      </c>
-      <c r="G442" s="2" t="inlineStr"/>
+        <v>56.15</v>
+      </c>
+      <c r="G442" s="3" t="n">
+        <v>18.87</v>
+      </c>
       <c r="H442" s="3" t="n">
-        <v>3.63</v>
+        <v>3.59</v>
       </c>
       <c r="I442" s="4" t="n">
-        <v>-0.0576</v>
+        <v>0.2184</v>
       </c>
       <c r="J442" s="4" t="n">
-        <v>-2.2771</v>
+        <v>-0.004500000000000001</v>
       </c>
       <c r="K442" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L442" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST ANA, BIST ANKARA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM TEMETTU, BIST KOCAELI, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
         </is>
       </c>
       <c r="M442" s="2" t="inlineStr"/>
@@ -19713,44 +19715,42 @@
     <row r="443">
       <c r="A443" s="6" t="inlineStr">
         <is>
-          <t>ARDYZ</t>
+          <t>EMKEL</t>
         </is>
       </c>
       <c r="B443" s="7" t="n">
-        <v>58</v>
+        <v>23.74</v>
       </c>
       <c r="C443" s="8" t="n">
-        <v>0.0184</v>
+        <v>-0.0389</v>
       </c>
       <c r="D443" s="9" t="n">
-        <v>5570000</v>
+        <v>11660000</v>
       </c>
       <c r="E443" s="8" t="n">
-        <v>0.3949</v>
+        <v>0.9773999999999999</v>
       </c>
       <c r="F443" s="7" t="n">
-        <v>64.19</v>
-      </c>
-      <c r="G443" s="7" t="n">
-        <v>27.7</v>
-      </c>
+        <v>46.43</v>
+      </c>
+      <c r="G443" s="6" t="inlineStr"/>
       <c r="H443" s="7" t="n">
-        <v>3.7</v>
+        <v>3.63</v>
       </c>
       <c r="I443" s="8" t="n">
-        <v>0.1333</v>
+        <v>-0.0576</v>
       </c>
       <c r="J443" s="8" t="n">
-        <v>6.844600000000001</v>
+        <v>-2.2771</v>
       </c>
       <c r="K443" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L443" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST ANA, BIST ANKARA</t>
         </is>
       </c>
       <c r="M443" s="6" t="inlineStr"/>
@@ -19758,42 +19758,44 @@
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>BARMA</t>
+          <t>ARDYZ</t>
         </is>
       </c>
       <c r="B444" s="3" t="n">
-        <v>61.2</v>
+        <v>58</v>
       </c>
       <c r="C444" s="4" t="n">
-        <v>0.0132</v>
+        <v>0.0184</v>
       </c>
       <c r="D444" s="5" t="n">
-        <v>3840000</v>
+        <v>5570000</v>
       </c>
       <c r="E444" s="4" t="n">
-        <v>0.2</v>
+        <v>0.3949</v>
       </c>
       <c r="F444" s="3" t="n">
-        <v>67.02</v>
-      </c>
-      <c r="G444" s="2" t="inlineStr"/>
+        <v>64.19</v>
+      </c>
+      <c r="G444" s="3" t="n">
+        <v>27.7</v>
+      </c>
       <c r="H444" s="3" t="n">
         <v>3.7</v>
       </c>
       <c r="I444" s="4" t="n">
-        <v>-0.005600000000000001</v>
+        <v>0.1333</v>
       </c>
       <c r="J444" s="4" t="n">
-        <v>-0.7101999999999999</v>
+        <v>6.844600000000001</v>
       </c>
       <c r="K444" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L444" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M444" s="2" t="inlineStr"/>
@@ -19801,44 +19803,42 @@
     <row r="445">
       <c r="A445" s="6" t="inlineStr">
         <is>
-          <t>PATEK</t>
+          <t>BARMA</t>
         </is>
       </c>
       <c r="B445" s="7" t="n">
-        <v>22.4</v>
+        <v>61.2</v>
       </c>
       <c r="C445" s="8" t="n">
-        <v>-0.0235</v>
+        <v>0.0132</v>
       </c>
       <c r="D445" s="9" t="n">
-        <v>47950000</v>
+        <v>3840000</v>
       </c>
       <c r="E445" s="8" t="n">
-        <v>0.4408</v>
+        <v>0.2</v>
       </c>
       <c r="F445" s="7" t="n">
-        <v>50.54</v>
-      </c>
-      <c r="G445" s="7" t="n">
-        <v>30.56</v>
-      </c>
+        <v>67.02</v>
+      </c>
+      <c r="G445" s="6" t="inlineStr"/>
       <c r="H445" s="7" t="n">
-        <v>3.81</v>
+        <v>3.7</v>
       </c>
       <c r="I445" s="8" t="n">
-        <v>0.1601</v>
+        <v>-0.005600000000000001</v>
       </c>
       <c r="J445" s="8" t="n">
-        <v>-6.4006</v>
+        <v>-0.7101999999999999</v>
       </c>
       <c r="K445" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L445" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST İZMİR</t>
         </is>
       </c>
       <c r="M445" s="6" t="inlineStr"/>
@@ -19846,42 +19846,44 @@
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>PAMEL</t>
+          <t>PATEK</t>
         </is>
       </c>
       <c r="B446" s="3" t="n">
-        <v>83.25</v>
+        <v>22.4</v>
       </c>
       <c r="C446" s="4" t="n">
-        <v>-0.0206</v>
+        <v>-0.0235</v>
       </c>
       <c r="D446" s="5" t="n">
-        <v>349050</v>
+        <v>47950000</v>
       </c>
       <c r="E446" s="4" t="n">
-        <v>0.2393</v>
+        <v>0.4408</v>
       </c>
       <c r="F446" s="3" t="n">
-        <v>41.59</v>
-      </c>
-      <c r="G446" s="2" t="inlineStr"/>
+        <v>50.54</v>
+      </c>
+      <c r="G446" s="3" t="n">
+        <v>30.56</v>
+      </c>
       <c r="H446" s="3" t="n">
-        <v>3.83</v>
+        <v>3.81</v>
       </c>
       <c r="I446" s="4" t="n">
-        <v>-0.4116</v>
+        <v>0.1601</v>
       </c>
       <c r="J446" s="4" t="n">
-        <v>-8.8185</v>
+        <v>-6.4006</v>
       </c>
       <c r="K446" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L446" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M446" s="2" t="inlineStr"/>
@@ -19889,42 +19891,42 @@
     <row r="447">
       <c r="A447" s="6" t="inlineStr">
         <is>
-          <t>OTTO</t>
+          <t>PAMEL</t>
         </is>
       </c>
       <c r="B447" s="7" t="n">
-        <v>286.25</v>
+        <v>83.25</v>
       </c>
       <c r="C447" s="8" t="n">
-        <v>-0.0394</v>
+        <v>-0.0206</v>
       </c>
       <c r="D447" s="9" t="n">
-        <v>357590</v>
+        <v>349050</v>
       </c>
       <c r="E447" s="8" t="n">
-        <v>0.3623</v>
+        <v>0.2393</v>
       </c>
       <c r="F447" s="7" t="n">
-        <v>33.59</v>
+        <v>41.59</v>
       </c>
       <c r="G447" s="6" t="inlineStr"/>
       <c r="H447" s="7" t="n">
-        <v>3.84</v>
+        <v>3.83</v>
       </c>
       <c r="I447" s="8" t="n">
-        <v>-0.0108</v>
+        <v>-0.4116</v>
       </c>
       <c r="J447" s="8" t="n">
-        <v>-0.3881</v>
+        <v>-8.8185</v>
       </c>
       <c r="K447" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L447" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST ANA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M447" s="6" t="inlineStr"/>
@@ -19932,33 +19934,33 @@
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>ALKA</t>
+          <t>OTTO</t>
         </is>
       </c>
       <c r="B448" s="3" t="n">
-        <v>10.95</v>
+        <v>286.25</v>
       </c>
       <c r="C448" s="4" t="n">
-        <v>-0.009899999999999999</v>
+        <v>-0.0394</v>
       </c>
       <c r="D448" s="5" t="n">
-        <v>8810000</v>
+        <v>357590</v>
       </c>
       <c r="E448" s="4" t="n">
-        <v>0.1937</v>
+        <v>0.3623</v>
       </c>
       <c r="F448" s="3" t="n">
-        <v>43.48</v>
+        <v>33.59</v>
       </c>
       <c r="G448" s="2" t="inlineStr"/>
       <c r="H448" s="3" t="n">
-        <v>3.87</v>
+        <v>3.84</v>
       </c>
       <c r="I448" s="4" t="n">
-        <v>-0.0556</v>
+        <v>-0.0108</v>
       </c>
       <c r="J448" s="4" t="n">
-        <v>-7.241000000000001</v>
+        <v>-0.3881</v>
       </c>
       <c r="K448" s="2" t="inlineStr">
         <is>
@@ -19967,7 +19969,7 @@
       </c>
       <c r="L448" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST ANA</t>
         </is>
       </c>
       <c r="M448" s="2" t="inlineStr"/>
@@ -19975,42 +19977,42 @@
     <row r="449">
       <c r="A449" s="6" t="inlineStr">
         <is>
-          <t>ALCAR</t>
+          <t>ALKA</t>
         </is>
       </c>
       <c r="B449" s="7" t="n">
-        <v>736.5</v>
+        <v>10.95</v>
       </c>
       <c r="C449" s="8" t="n">
-        <v>-0.0379</v>
+        <v>-0.009899999999999999</v>
       </c>
       <c r="D449" s="9" t="n">
-        <v>42960</v>
+        <v>8810000</v>
       </c>
       <c r="E449" s="8" t="n">
-        <v>0.1594</v>
+        <v>0.1937</v>
       </c>
       <c r="F449" s="7" t="n">
-        <v>38.06</v>
+        <v>43.48</v>
       </c>
       <c r="G449" s="6" t="inlineStr"/>
       <c r="H449" s="7" t="n">
-        <v>3.91</v>
+        <v>3.87</v>
       </c>
       <c r="I449" s="8" t="n">
-        <v>-0.2165</v>
+        <v>-0.0556</v>
       </c>
       <c r="J449" s="8" t="n">
-        <v>0.7798999999999999</v>
+        <v>-7.241000000000001</v>
       </c>
       <c r="K449" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L449" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST İSTANBUL, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M449" s="6" t="inlineStr"/>
@@ -20018,35 +20020,33 @@
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>EUPWR</t>
+          <t>ALCAR</t>
         </is>
       </c>
       <c r="B450" s="3" t="n">
-        <v>62.55</v>
+        <v>736.5</v>
       </c>
       <c r="C450" s="4" t="n">
-        <v>0.0279</v>
+        <v>-0.0379</v>
       </c>
       <c r="D450" s="5" t="n">
-        <v>28820000</v>
+        <v>42960</v>
       </c>
       <c r="E450" s="4" t="n">
-        <v>0.3025</v>
+        <v>0.1594</v>
       </c>
       <c r="F450" s="3" t="n">
-        <v>70.98999999999999</v>
-      </c>
-      <c r="G450" s="3" t="n">
-        <v>72.01000000000001</v>
-      </c>
+        <v>38.06</v>
+      </c>
+      <c r="G450" s="2" t="inlineStr"/>
       <c r="H450" s="3" t="n">
-        <v>3.92</v>
+        <v>3.91</v>
       </c>
       <c r="I450" s="4" t="n">
-        <v>0.06320000000000001</v>
+        <v>-0.2165</v>
       </c>
       <c r="J450" s="4" t="n">
-        <v>-1.0812</v>
+        <v>0.7798999999999999</v>
       </c>
       <c r="K450" s="2" t="inlineStr">
         <is>
@@ -20055,7 +20055,7 @@
       </c>
       <c r="L450" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST İSTANBUL, BIST ANA</t>
         </is>
       </c>
       <c r="M450" s="2" t="inlineStr"/>
@@ -20063,42 +20063,44 @@
     <row r="451">
       <c r="A451" s="6" t="inlineStr">
         <is>
-          <t>ENSRI</t>
+          <t>EUPWR</t>
         </is>
       </c>
       <c r="B451" s="7" t="n">
-        <v>10.2</v>
+        <v>62.55</v>
       </c>
       <c r="C451" s="8" t="n">
-        <v>0.0241</v>
+        <v>0.0279</v>
       </c>
       <c r="D451" s="9" t="n">
-        <v>101230000</v>
+        <v>28820000</v>
       </c>
       <c r="E451" s="8" t="n">
-        <v>0.4329</v>
+        <v>0.3025</v>
       </c>
       <c r="F451" s="7" t="n">
-        <v>24.49</v>
-      </c>
-      <c r="G451" s="6" t="inlineStr"/>
+        <v>70.98999999999999</v>
+      </c>
+      <c r="G451" s="7" t="n">
+        <v>72.01000000000001</v>
+      </c>
       <c r="H451" s="7" t="n">
-        <v>3.94</v>
+        <v>3.92</v>
       </c>
       <c r="I451" s="8" t="n">
-        <v>-0.0555</v>
+        <v>0.06320000000000001</v>
       </c>
       <c r="J451" s="8" t="n">
-        <v>-10.8224</v>
+        <v>-1.0812</v>
       </c>
       <c r="K451" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L451" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M451" s="6" t="inlineStr"/>
@@ -20106,44 +20108,42 @@
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>LOGO</t>
+          <t>ENSRI</t>
         </is>
       </c>
       <c r="B452" s="3" t="n">
-        <v>155</v>
+        <v>10.2</v>
       </c>
       <c r="C452" s="4" t="n">
-        <v>-0.0252</v>
+        <v>0.0241</v>
       </c>
       <c r="D452" s="5" t="n">
-        <v>1190000</v>
+        <v>101230000</v>
       </c>
       <c r="E452" s="4" t="n">
-        <v>0.6459999999999999</v>
+        <v>0.4329</v>
       </c>
       <c r="F452" s="3" t="n">
-        <v>56.15</v>
-      </c>
-      <c r="G452" s="3" t="n">
-        <v>10.61</v>
-      </c>
+        <v>24.49</v>
+      </c>
+      <c r="G452" s="2" t="inlineStr"/>
       <c r="H452" s="3" t="n">
         <v>3.94</v>
       </c>
       <c r="I452" s="4" t="n">
-        <v>0.4715</v>
+        <v>-0.0555</v>
       </c>
       <c r="J452" s="4" t="n">
-        <v>-0.4521</v>
+        <v>-10.8224</v>
       </c>
       <c r="K452" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L452" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM TEMETTU, BIST KOCAELI, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M452" s="2" t="inlineStr"/>
@@ -25911,34 +25911,38 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>13.96</v>
+        <v>65.15000000000001</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.0285</v>
+        <v>-0.0585</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>30370000</v>
-      </c>
-      <c r="E587" s="6" t="inlineStr"/>
+        <v>869750</v>
+      </c>
+      <c r="E587" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F587" s="7" t="n">
-        <v>49.07</v>
+        <v>49.58</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
       <c r="I587" s="6" t="inlineStr"/>
-      <c r="J587" s="6" t="inlineStr"/>
+      <c r="J587" s="8" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25981,87 +25985,95 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>69.09999999999999</v>
+        <v>6.44</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0162</v>
+        <v>0.0733</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>48030</v>
+        <v>19120000</v>
       </c>
       <c r="E589" s="8" t="n">
-        <v>0.58</v>
+        <v>0.8667</v>
       </c>
       <c r="F589" s="7" t="n">
-        <v>36.59</v>
+        <v>70.31</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J589" s="8" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I589" s="6" t="inlineStr"/>
+      <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>78.62</v>
+        <v>13.96</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0067</v>
+        <v>-0.0285</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>11350000</v>
+        <v>30370000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>37.39</v>
+        <v>49.07</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="2" t="inlineStr"/>
       <c r="J590" s="2" t="inlineStr"/>
-      <c r="K590" s="2" t="inlineStr"/>
-      <c r="L590" s="2" t="inlineStr"/>
+      <c r="K590" s="2" t="inlineStr">
+        <is>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>240.1</v>
+        <v>30.64</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.02</v>
+        <v>-0.07820000000000001</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>10620</v>
+        <v>16140000</v>
       </c>
       <c r="E591" s="8" t="n">
-        <v>0.2578</v>
+        <v>0.2667</v>
       </c>
       <c r="F591" s="7" t="n">
-        <v>43.77</v>
+        <v>52.53</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26069,30 +26081,34 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>77.25</v>
+        <v>28.4</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.09960000000000001</v>
+        <v>-0.0373</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>29900000</v>
+        <v>23640000</v>
       </c>
       <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>88.89</v>
+        <v>55.6</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26100,12 +26116,12 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26113,58 +26129,56 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>9.93</v>
+        <v>42.32</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.0793</v>
+        <v>0.0272</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>757940</v>
-      </c>
-      <c r="E593" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>5980000</v>
+      </c>
+      <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>61.27</v>
+        <v>53.18</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J593" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I593" s="6" t="inlineStr"/>
+      <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>2.73</v>
+        <v>6.06</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>142720000</v>
+        <v>7340000</v>
       </c>
       <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>45.93</v>
+        <v>45.24</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26175,74 +26189,64 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L594" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+      <c r="L594" s="2" t="inlineStr"/>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>2.48</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.008</v>
+        <v>0.0162</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>21880000</v>
+        <v>48030</v>
       </c>
       <c r="E595" s="8" t="n">
-        <v>1</v>
+        <v>0.58</v>
       </c>
       <c r="F595" s="7" t="n">
-        <v>35.12</v>
+        <v>36.59</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="8" t="n">
-        <v>-191.6342</v>
+        <v>-9.409700000000001</v>
       </c>
       <c r="J595" s="8" t="n">
-        <v>-0.8093</v>
+        <v>-4.155</v>
       </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr"/>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>6.44</v>
+        <v>36.4</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0733</v>
+        <v>0.0196</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>19120000</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>6480000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>70.31</v>
+        <v>58.24</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26250,12 +26254,12 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26263,56 +26267,58 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>198.4</v>
+        <v>9.93</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0345</v>
+        <v>0.0793</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>8520000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>757940</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>61.52</v>
+        <v>61.27</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>42.32</v>
+        <v>73.8</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.0272</v>
+        <v>-0.0238</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>5980000</v>
+        <v>174630</v>
       </c>
       <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>53.18</v>
+        <v>10.48</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26320,51 +26326,43 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L598" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr"/>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>65.15000000000001</v>
+        <v>2.73</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0585</v>
+        <v>0</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>869750</v>
-      </c>
-      <c r="E599" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>142720000</v>
+      </c>
+      <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>49.58</v>
+        <v>45.93</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
       <c r="I599" s="6" t="inlineStr"/>
-      <c r="J599" s="8" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26372,26 +26370,32 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>18.53</v>
+        <v>5.97</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0011</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>55440000</v>
-      </c>
-      <c r="E600" s="2" t="inlineStr"/>
+        <v>35800000</v>
+      </c>
+      <c r="E600" s="4" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F600" s="3" t="n">
-        <v>35.89</v>
+        <v>49.23</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="2" t="inlineStr"/>
-      <c r="J600" s="2" t="inlineStr"/>
+      <c r="I600" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J600" s="4" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26399,7 +26403,7 @@
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26407,40 +26411,42 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>5.97</v>
+        <v>34.68</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.09939999999999999</v>
+        <v>-0.0181</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>35800000</v>
+        <v>5190000</v>
       </c>
       <c r="E601" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.3528</v>
       </c>
       <c r="F601" s="7" t="n">
-        <v>49.23</v>
-      </c>
-      <c r="G601" s="6" t="inlineStr"/>
+        <v>43.26</v>
+      </c>
+      <c r="G601" s="7" t="n">
+        <v>13.71</v>
+      </c>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="8" t="n">
-        <v>-5.3262</v>
+        <v>0.1029</v>
       </c>
       <c r="J601" s="8" t="n">
-        <v>-4.2562</v>
+        <v>-1.4864</v>
       </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26448,114 +26454,108 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>142.7</v>
+        <v>240.1</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.061</v>
+        <v>-0.02</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>995180</v>
+        <v>10620</v>
       </c>
       <c r="E602" s="4" t="n">
-        <v>0.1071</v>
+        <v>0.2578</v>
       </c>
       <c r="F602" s="3" t="n">
-        <v>48.18</v>
+        <v>43.77</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J602" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I602" s="2" t="inlineStr"/>
+      <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr"/>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>73.8</v>
+        <v>142.7</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0238</v>
+        <v>0.061</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>174630</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>995180</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>10.48</v>
+        <v>48.18</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="6" t="inlineStr"/>
+      <c r="I603" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J603" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr"/>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>34.68</v>
+        <v>17.05</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0181</v>
+        <v>-0.0512</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>5190000</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>48680000</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>43.26</v>
-      </c>
-      <c r="G604" s="3" t="n">
-        <v>13.71</v>
-      </c>
+        <v>49.01</v>
+      </c>
+      <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="4" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J604" s="4" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I604" s="2" t="inlineStr"/>
+      <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26563,36 +26563,40 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>30.64</v>
+        <v>2.48</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.07820000000000001</v>
+        <v>-0.008</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>16140000</v>
+        <v>21880000</v>
       </c>
       <c r="E605" s="8" t="n">
-        <v>0.2667</v>
+        <v>1</v>
       </c>
       <c r="F605" s="7" t="n">
-        <v>52.53</v>
+        <v>35.12</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="6" t="inlineStr"/>
-      <c r="J605" s="6" t="inlineStr"/>
+      <c r="I605" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J605" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26600,21 +26604,21 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>6.06</v>
+        <v>77.25</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.008199999999999999</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>7340000</v>
+        <v>29900000</v>
       </c>
       <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>45.24</v>
+        <v>88.89</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26622,43 +26626,51 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr"/>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>178.6</v>
+        <v>26.02</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0341</v>
+        <v>-0.008399999999999999</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>8620000</v>
-      </c>
-      <c r="E607" s="6" t="inlineStr"/>
+        <v>883760</v>
+      </c>
+      <c r="E607" s="8" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F607" s="7" t="n">
-        <v>38.77</v>
+        <v>43.34</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
       <c r="I607" s="6" t="inlineStr"/>
-      <c r="J607" s="6" t="inlineStr"/>
+      <c r="J607" s="8" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26666,21 +26678,21 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>36.4</v>
+        <v>178.6</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0196</v>
+        <v>-0.0341</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>6480000</v>
+        <v>8620000</v>
       </c>
       <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>58.24</v>
+        <v>38.77</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
@@ -26688,12 +26700,12 @@
       <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26701,38 +26713,34 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>26.02</v>
+        <v>18.53</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>-0.008399999999999999</v>
+        <v>0.0011</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>883760</v>
-      </c>
-      <c r="E609" s="8" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>55440000</v>
+      </c>
+      <c r="E609" s="6" t="inlineStr"/>
       <c r="F609" s="7" t="n">
-        <v>43.34</v>
+        <v>35.89</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
       <c r="I609" s="6" t="inlineStr"/>
-      <c r="J609" s="8" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J609" s="6" t="inlineStr"/>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26740,21 +26748,21 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>17.05</v>
+        <v>198.4</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.0512</v>
+        <v>-0.0345</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>48680000</v>
+        <v>8520000</v>
       </c>
       <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>49.01</v>
+        <v>61.52</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
@@ -26762,12 +26770,12 @@
       <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M610" s="2" t="inlineStr"/>
@@ -26775,36 +26783,28 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>28.4</v>
+        <v>78.62</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.0373</v>
+        <v>-0.0067</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>23640000</v>
+        <v>11350000</v>
       </c>
       <c r="E611" s="6" t="inlineStr"/>
       <c r="F611" s="7" t="n">
-        <v>55.6</v>
+        <v>37.39</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
       <c r="I611" s="6" t="inlineStr"/>
       <c r="J611" s="6" t="inlineStr"/>
-      <c r="K611" s="6" t="inlineStr">
-        <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L611" s="6" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+      <c r="K611" s="6" t="inlineStr"/>
+      <c r="L611" s="6" t="inlineStr"/>
       <c r="M611" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26829,7 +26829,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>19.05.2026 12:30</t>
+          <t>19.05.2026 13:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 19.05.2026 14:30 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-19.xlsx
+++ b/data/bist_screener_2026-05-19.xlsx
@@ -25911,60 +25911,60 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>65.15000000000001</v>
+        <v>9.93</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.0585</v>
+        <v>0.0793</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>869750</v>
+        <v>757940</v>
       </c>
       <c r="E587" s="8" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.95</v>
       </c>
       <c r="F587" s="7" t="n">
-        <v>49.58</v>
+        <v>61.27</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="6" t="inlineStr"/>
+      <c r="I587" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
       <c r="J587" s="8" t="n">
-        <v>0.1431</v>
+        <v>-0.4678</v>
       </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
-        </is>
-      </c>
-      <c r="L587" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L587" s="6" t="inlineStr"/>
       <c r="M587" s="6" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>18.16</v>
+        <v>6.44</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0145</v>
+        <v>0.0733</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>45490000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>19120000</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>52.57</v>
+        <v>70.31</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25972,12 +25972,12 @@
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25985,23 +25985,21 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>6.44</v>
+        <v>198.4</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0733</v>
+        <v>-0.0345</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>19120000</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>8520000</v>
+      </c>
+      <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>70.31</v>
+        <v>61.52</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26009,12 +26007,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26022,21 +26020,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>13.96</v>
+        <v>77.25</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0285</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>30370000</v>
+        <v>29900000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>49.07</v>
+        <v>88.89</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26044,12 +26042,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26057,23 +26055,21 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>30.64</v>
+        <v>42.32</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.07820000000000001</v>
+        <v>0.0272</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>16140000</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>5980000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>52.53</v>
+        <v>53.18</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26081,12 +26077,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26094,34 +26090,40 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>28.4</v>
+        <v>2.48</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0373</v>
+        <v>-0.008</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>23640000</v>
-      </c>
-      <c r="E592" s="2" t="inlineStr"/>
+        <v>21880000</v>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="F592" s="3" t="n">
-        <v>55.6</v>
+        <v>35.12</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="2" t="inlineStr"/>
+      <c r="I592" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J592" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26129,21 +26131,21 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>42.32</v>
+        <v>73.8</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.0272</v>
+        <v>-0.0238</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>5980000</v>
+        <v>174630</v>
       </c>
       <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>53.18</v>
+        <v>10.48</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
@@ -26151,205 +26153,213 @@
       <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr"/>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>6.06</v>
+        <v>142.7</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.008199999999999999</v>
+        <v>0.061</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>7340000</v>
-      </c>
-      <c r="E594" s="2" t="inlineStr"/>
+        <v>995180</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F594" s="3" t="n">
-        <v>45.24</v>
+        <v>48.18</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="I594" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J594" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr"/>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>69.09999999999999</v>
+        <v>18.53</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0162</v>
+        <v>0.0011</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>48030</v>
-      </c>
-      <c r="E595" s="8" t="n">
-        <v>0.58</v>
-      </c>
+        <v>55440000</v>
+      </c>
+      <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>36.59</v>
+        <v>35.89</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J595" s="8" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I595" s="6" t="inlineStr"/>
+      <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>36.4</v>
+        <v>78.62</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0196</v>
+        <v>-0.0067</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>6480000</v>
+        <v>11350000</v>
       </c>
       <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>58.24</v>
+        <v>37.39</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
       <c r="I596" s="2" t="inlineStr"/>
       <c r="J596" s="2" t="inlineStr"/>
-      <c r="K596" s="2" t="inlineStr">
-        <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+      <c r="K596" s="2" t="inlineStr"/>
+      <c r="L596" s="2" t="inlineStr"/>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>9.93</v>
+        <v>5.97</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0793</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>757940</v>
+        <v>35800000</v>
       </c>
       <c r="E597" s="8" t="n">
-        <v>0.95</v>
+        <v>0.1672</v>
       </c>
       <c r="F597" s="7" t="n">
-        <v>61.27</v>
+        <v>49.23</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
       <c r="I597" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-5.3262</v>
       </c>
       <c r="J597" s="8" t="n">
-        <v>-0.4678</v>
+        <v>-4.2562</v>
       </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>73.8</v>
+        <v>65.15000000000001</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0238</v>
+        <v>-0.0585</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>174630</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>869750</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>10.48</v>
+        <v>49.58</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="2" t="inlineStr"/>
+      <c r="J598" s="4" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L598" s="2" t="inlineStr"/>
+          <t>Teknoloji hizmetleri</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>2.73</v>
+        <v>13.96</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0</v>
+        <v>-0.0285</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>142720000</v>
+        <v>30370000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>45.93</v>
+        <v>49.07</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26357,12 +26367,12 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26370,40 +26380,34 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>5.97</v>
+        <v>28.4</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.09939999999999999</v>
+        <v>-0.0373</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>35800000</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>23640000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>49.23</v>
+        <v>55.6</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J600" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I600" s="2" t="inlineStr"/>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26411,42 +26415,34 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>34.68</v>
+        <v>36.4</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0181</v>
+        <v>0.0196</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>5190000</v>
-      </c>
-      <c r="E601" s="8" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>6480000</v>
+      </c>
+      <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>43.26</v>
-      </c>
-      <c r="G601" s="7" t="n">
-        <v>13.71</v>
-      </c>
+        <v>58.24</v>
+      </c>
+      <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J601" s="8" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26454,23 +26450,21 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>240.1</v>
+        <v>17.05</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.02</v>
+        <v>-0.0512</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>10620</v>
-      </c>
-      <c r="E602" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>48680000</v>
+      </c>
+      <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>43.77</v>
+        <v>49.01</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26478,49 +26472,47 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>142.7</v>
+        <v>178.6</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.061</v>
+        <v>-0.0341</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>995180</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>8620000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>48.18</v>
+        <v>38.77</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26528,34 +26520,38 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>17.05</v>
+        <v>26.02</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0512</v>
+        <v>-0.008399999999999999</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>48680000</v>
-      </c>
-      <c r="E604" s="2" t="inlineStr"/>
+        <v>883760</v>
+      </c>
+      <c r="E604" s="4" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F604" s="3" t="n">
-        <v>49.01</v>
+        <v>43.34</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
       <c r="I604" s="2" t="inlineStr"/>
-      <c r="J604" s="2" t="inlineStr"/>
+      <c r="J604" s="4" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26563,62 +26559,54 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>2.48</v>
+        <v>6.06</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.008</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>21880000</v>
-      </c>
-      <c r="E605" s="8" t="n">
-        <v>1</v>
-      </c>
+        <v>7340000</v>
+      </c>
+      <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>35.12</v>
+        <v>45.24</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J605" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I605" s="6" t="inlineStr"/>
+      <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L605" s="6" t="inlineStr"/>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>77.25</v>
+        <v>240.1</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.09960000000000001</v>
+        <v>-0.02</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>29900000</v>
-      </c>
-      <c r="E606" s="2" t="inlineStr"/>
+        <v>10620</v>
+      </c>
+      <c r="E606" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F606" s="3" t="n">
-        <v>88.89</v>
+        <v>43.77</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26626,42 +26614,42 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr"/>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>26.02</v>
+        <v>34.68</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.008399999999999999</v>
+        <v>-0.0181</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>883760</v>
+        <v>5190000</v>
       </c>
       <c r="E607" s="8" t="n">
-        <v>0.9698</v>
+        <v>0.3528</v>
       </c>
       <c r="F607" s="7" t="n">
-        <v>43.34</v>
-      </c>
-      <c r="G607" s="6" t="inlineStr"/>
+        <v>43.26</v>
+      </c>
+      <c r="G607" s="7" t="n">
+        <v>13.71</v>
+      </c>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="6" t="inlineStr"/>
+      <c r="I607" s="8" t="n">
+        <v>0.1029</v>
+      </c>
       <c r="J607" s="8" t="n">
-        <v>0.6453</v>
+        <v>-1.4864</v>
       </c>
       <c r="K607" s="6" t="inlineStr">
         <is>
@@ -26670,7 +26658,7 @@
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26678,56 +26666,58 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>178.6</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>-0.0341</v>
+        <v>0.0162</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>8620000</v>
-      </c>
-      <c r="E608" s="2" t="inlineStr"/>
+        <v>48030</v>
+      </c>
+      <c r="E608" s="4" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F608" s="3" t="n">
-        <v>38.77</v>
+        <v>36.59</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
-      <c r="I608" s="2" t="inlineStr"/>
-      <c r="J608" s="2" t="inlineStr"/>
+      <c r="I608" s="4" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J608" s="4" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L608" s="2" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L608" s="2" t="inlineStr"/>
       <c r="M608" s="2" t="inlineStr"/>
     </row>
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>18.53</v>
+        <v>18.16</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0145</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>55440000</v>
+        <v>45490000</v>
       </c>
       <c r="E609" s="6" t="inlineStr"/>
       <c r="F609" s="7" t="n">
-        <v>35.89</v>
+        <v>52.57</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
@@ -26735,12 +26725,12 @@
       <c r="J609" s="6" t="inlineStr"/>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26748,21 +26738,23 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>198.4</v>
+        <v>30.64</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.0345</v>
+        <v>-0.07820000000000001</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>8520000</v>
-      </c>
-      <c r="E610" s="2" t="inlineStr"/>
+        <v>16140000</v>
+      </c>
+      <c r="E610" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F610" s="3" t="n">
-        <v>61.52</v>
+        <v>52.53</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
@@ -26770,12 +26762,12 @@
       <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M610" s="2" t="inlineStr"/>
@@ -26783,28 +26775,36 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>78.62</v>
+        <v>2.73</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.0067</v>
+        <v>0</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>11350000</v>
+        <v>142720000</v>
       </c>
       <c r="E611" s="6" t="inlineStr"/>
       <c r="F611" s="7" t="n">
-        <v>37.39</v>
+        <v>45.93</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
       <c r="I611" s="6" t="inlineStr"/>
       <c r="J611" s="6" t="inlineStr"/>
-      <c r="K611" s="6" t="inlineStr"/>
-      <c r="L611" s="6" t="inlineStr"/>
+      <c r="K611" s="6" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L611" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M611" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26829,7 +26829,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>19.05.2026 13:30</t>
+          <t>19.05.2026 14:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 19.05.2026 15:30 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-19.xlsx
+++ b/data/bist_screener_2026-05-19.xlsx
@@ -25911,60 +25911,62 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>9.93</v>
+        <v>2.48</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0793</v>
+        <v>-0.008</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>757940</v>
+        <v>21880000</v>
       </c>
       <c r="E587" s="8" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="F587" s="7" t="n">
-        <v>61.27</v>
+        <v>35.12</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
       <c r="I587" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-191.6342</v>
       </c>
       <c r="J587" s="8" t="n">
-        <v>-0.4678</v>
+        <v>-0.8093</v>
       </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L587" s="6" t="inlineStr"/>
+          <t>Dağıtım servisleri</t>
+        </is>
+      </c>
+      <c r="L587" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M587" s="6" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>6.44</v>
+        <v>42.32</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0733</v>
+        <v>0.0272</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>19120000</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>5980000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>70.31</v>
+        <v>53.18</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25972,12 +25974,12 @@
       <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25985,21 +25987,21 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>198.4</v>
+        <v>17.05</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0345</v>
+        <v>-0.0512</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>8520000</v>
+        <v>48680000</v>
       </c>
       <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>61.52</v>
+        <v>49.01</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26007,12 +26009,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26020,21 +26022,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>77.25</v>
+        <v>73.8</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.09960000000000001</v>
+        <v>-0.0238</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>29900000</v>
+        <v>174630</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>88.89</v>
+        <v>10.48</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26042,34 +26044,30 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L590" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr"/>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>42.32</v>
+        <v>36.4</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0272</v>
+        <v>0.0196</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>5980000</v>
+        <v>6480000</v>
       </c>
       <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>53.18</v>
+        <v>58.24</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26077,12 +26075,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26090,112 +26088,98 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>2.48</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.008</v>
+        <v>0.0162</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>21880000</v>
+        <v>48030</v>
       </c>
       <c r="E592" s="4" t="n">
-        <v>1</v>
+        <v>0.58</v>
       </c>
       <c r="F592" s="3" t="n">
-        <v>35.12</v>
+        <v>36.59</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
       <c r="I592" s="4" t="n">
-        <v>-191.6342</v>
+        <v>-9.409700000000001</v>
       </c>
       <c r="J592" s="4" t="n">
-        <v>-0.8093</v>
+        <v>-4.155</v>
       </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr"/>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>73.8</v>
+        <v>78.62</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0238</v>
+        <v>-0.0067</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>174630</v>
+        <v>11350000</v>
       </c>
       <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>10.48</v>
+        <v>37.39</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
       <c r="I593" s="6" t="inlineStr"/>
       <c r="J593" s="6" t="inlineStr"/>
-      <c r="K593" s="6" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
+      <c r="K593" s="6" t="inlineStr"/>
       <c r="L593" s="6" t="inlineStr"/>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>142.7</v>
+        <v>13.96</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.061</v>
+        <v>-0.0285</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>995180</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>30370000</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>48.18</v>
+        <v>49.07</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J594" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I594" s="2" t="inlineStr"/>
+      <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26203,21 +26187,21 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>18.53</v>
+        <v>77.25</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>55440000</v>
+        <v>29900000</v>
       </c>
       <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>35.89</v>
+        <v>88.89</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
@@ -26225,12 +26209,12 @@
       <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26238,28 +26222,42 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>78.62</v>
+        <v>142.7</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0067</v>
+        <v>0.061</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>11350000</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>995180</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>37.39</v>
+        <v>48.18</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="2" t="inlineStr"/>
-      <c r="K596" s="2" t="inlineStr"/>
-      <c r="L596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J596" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
+      <c r="K596" s="2" t="inlineStr">
+        <is>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
@@ -26306,38 +26304,38 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>65.15000000000001</v>
+        <v>26.02</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0585</v>
+        <v>-0.008399999999999999</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>869750</v>
+        <v>883760</v>
       </c>
       <c r="E598" s="4" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.9698</v>
       </c>
       <c r="F598" s="3" t="n">
-        <v>49.58</v>
+        <v>43.34</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
       <c r="J598" s="4" t="n">
-        <v>0.1431</v>
+        <v>0.6453</v>
       </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26345,21 +26343,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>13.96</v>
+        <v>18.16</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0285</v>
+        <v>0.0145</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>30370000</v>
+        <v>45490000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>49.07</v>
+        <v>52.57</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26367,12 +26365,12 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26380,34 +26378,42 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>28.4</v>
+        <v>34.68</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.0373</v>
+        <v>-0.0181</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>23640000</v>
-      </c>
-      <c r="E600" s="2" t="inlineStr"/>
+        <v>5190000</v>
+      </c>
+      <c r="E600" s="4" t="n">
+        <v>0.3528</v>
+      </c>
       <c r="F600" s="3" t="n">
-        <v>55.6</v>
-      </c>
-      <c r="G600" s="2" t="inlineStr"/>
+        <v>43.26</v>
+      </c>
+      <c r="G600" s="3" t="n">
+        <v>13.71</v>
+      </c>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="2" t="inlineStr"/>
-      <c r="J600" s="2" t="inlineStr"/>
+      <c r="I600" s="4" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J600" s="4" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26415,21 +26421,23 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>36.4</v>
+        <v>240.1</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0196</v>
+        <v>-0.02</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>6480000</v>
-      </c>
-      <c r="E601" s="6" t="inlineStr"/>
+        <v>10620</v>
+      </c>
+      <c r="E601" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F601" s="7" t="n">
-        <v>58.24</v>
+        <v>43.77</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
@@ -26437,34 +26445,30 @@
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>17.05</v>
+        <v>2.73</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0512</v>
+        <v>0</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>48680000</v>
+        <v>142720000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>49.01</v>
+        <v>45.93</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26477,7 +26481,7 @@
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26485,34 +26489,38 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>178.6</v>
+        <v>65.15000000000001</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0341</v>
+        <v>-0.0585</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>8620000</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>869750</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>38.77</v>
+        <v>49.58</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
       <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="6" t="inlineStr"/>
+      <c r="J603" s="8" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26520,38 +26528,34 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>26.02</v>
+        <v>198.4</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.008399999999999999</v>
+        <v>-0.0345</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>883760</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>8520000</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>43.34</v>
+        <v>61.52</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
       <c r="I604" s="2" t="inlineStr"/>
-      <c r="J604" s="4" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26559,21 +26563,21 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>6.06</v>
+        <v>178.6</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.008199999999999999</v>
+        <v>-0.0341</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>7340000</v>
+        <v>8620000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>45.24</v>
+        <v>38.77</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26581,32 +26585,36 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L605" s="6" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>240.1</v>
+        <v>6.44</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.02</v>
+        <v>0.0733</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>10620</v>
+        <v>19120000</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.2578</v>
+        <v>0.8667</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>43.77</v>
+        <v>70.31</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26614,51 +26622,47 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>34.68</v>
+        <v>18.53</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0181</v>
+        <v>0.0011</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>5190000</v>
-      </c>
-      <c r="E607" s="8" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>55440000</v>
+      </c>
+      <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>43.26</v>
-      </c>
-      <c r="G607" s="7" t="n">
-        <v>13.71</v>
-      </c>
+        <v>35.89</v>
+      </c>
+      <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="8" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J607" s="8" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I607" s="6" t="inlineStr"/>
+      <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26666,58 +26670,56 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>69.09999999999999</v>
+        <v>28.4</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0162</v>
+        <v>-0.0373</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>48030</v>
-      </c>
-      <c r="E608" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>23640000</v>
+      </c>
+      <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>36.59</v>
+        <v>55.6</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
-      <c r="I608" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J608" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I608" s="2" t="inlineStr"/>
+      <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L608" s="2" t="inlineStr"/>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
+        </is>
+      </c>
+      <c r="L608" s="2" t="inlineStr">
+        <is>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M608" s="2" t="inlineStr"/>
     </row>
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>18.16</v>
+        <v>6.06</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.0145</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>45490000</v>
+        <v>7340000</v>
       </c>
       <c r="E609" s="6" t="inlineStr"/>
       <c r="F609" s="7" t="n">
-        <v>52.57</v>
+        <v>45.24</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
@@ -26725,71 +26727,69 @@
       <c r="J609" s="6" t="inlineStr"/>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L609" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L609" s="6" t="inlineStr"/>
       <c r="M609" s="6" t="inlineStr"/>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>30.64</v>
+        <v>9.93</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.07820000000000001</v>
+        <v>0.0793</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>16140000</v>
+        <v>757940</v>
       </c>
       <c r="E610" s="4" t="n">
-        <v>0.2667</v>
+        <v>0.95</v>
       </c>
       <c r="F610" s="3" t="n">
-        <v>52.53</v>
+        <v>61.27</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
-      <c r="I610" s="2" t="inlineStr"/>
-      <c r="J610" s="2" t="inlineStr"/>
+      <c r="I610" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J610" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L610" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L610" s="2" t="inlineStr"/>
       <c r="M610" s="2" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>2.73</v>
+        <v>30.64</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>0</v>
+        <v>-0.07820000000000001</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>142720000</v>
-      </c>
-      <c r="E611" s="6" t="inlineStr"/>
+        <v>16140000</v>
+      </c>
+      <c r="E611" s="8" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F611" s="7" t="n">
-        <v>45.93</v>
+        <v>52.53</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
@@ -26797,12 +26797,12 @@
       <c r="J611" s="6" t="inlineStr"/>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26829,7 +26829,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>19.05.2026 14:30</t>
+          <t>19.05.2026 15:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 19.05.2026 16:30 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-19.xlsx
+++ b/data/bist_screener_2026-05-19.xlsx
@@ -25911,97 +25911,91 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>2.48</v>
+        <v>240.1</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.008</v>
+        <v>-0.02</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>21880000</v>
+        <v>10620</v>
       </c>
       <c r="E587" s="8" t="n">
-        <v>1</v>
+        <v>0.2578</v>
       </c>
       <c r="F587" s="7" t="n">
-        <v>35.12</v>
+        <v>43.77</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J587" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I587" s="6" t="inlineStr"/>
+      <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
-        </is>
-      </c>
-      <c r="L587" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L587" s="6" t="inlineStr"/>
       <c r="M587" s="6" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>42.32</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0272</v>
+        <v>0.0162</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>5980000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>48030</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>53.18</v>
+        <v>36.59</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="I588" s="4" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J588" s="4" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L588" s="2" t="inlineStr"/>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>17.05</v>
+        <v>28.4</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0512</v>
+        <v>-0.0373</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>48680000</v>
+        <v>23640000</v>
       </c>
       <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>49.01</v>
+        <v>55.6</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26009,12 +26003,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26022,21 +26016,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>73.8</v>
+        <v>178.6</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0238</v>
+        <v>-0.0341</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>174630</v>
+        <v>8620000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>10.48</v>
+        <v>38.77</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26044,43 +26038,51 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L590" s="2" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>36.4</v>
+        <v>26.02</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0196</v>
+        <v>-0.008399999999999999</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>6480000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>883760</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>58.24</v>
+        <v>43.34</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
       <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="6" t="inlineStr"/>
+      <c r="J591" s="8" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26088,98 +26090,110 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>69.09999999999999</v>
+        <v>13.96</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0162</v>
+        <v>-0.0285</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>48030</v>
-      </c>
-      <c r="E592" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>30370000</v>
+      </c>
+      <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>36.59</v>
+        <v>49.07</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J592" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I592" s="2" t="inlineStr"/>
+      <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr"/>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>78.62</v>
+        <v>36.4</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0067</v>
+        <v>0.0196</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>11350000</v>
+        <v>6480000</v>
       </c>
       <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>37.39</v>
+        <v>58.24</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
       <c r="I593" s="6" t="inlineStr"/>
       <c r="J593" s="6" t="inlineStr"/>
-      <c r="K593" s="6" t="inlineStr"/>
-      <c r="L593" s="6" t="inlineStr"/>
+      <c r="K593" s="6" t="inlineStr">
+        <is>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>13.96</v>
+        <v>2.48</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0285</v>
+        <v>-0.008</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>30370000</v>
-      </c>
-      <c r="E594" s="2" t="inlineStr"/>
+        <v>21880000</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="F594" s="3" t="n">
-        <v>49.07</v>
+        <v>35.12</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="I594" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J594" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26187,21 +26201,21 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>77.25</v>
+        <v>18.16</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.09960000000000001</v>
+        <v>0.0145</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>29900000</v>
+        <v>45490000</v>
       </c>
       <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>88.89</v>
+        <v>52.57</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
@@ -26209,12 +26223,12 @@
       <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26222,40 +26236,40 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>142.7</v>
+        <v>5.97</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.061</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>995180</v>
+        <v>35800000</v>
       </c>
       <c r="E596" s="4" t="n">
-        <v>0.1071</v>
+        <v>0.1672</v>
       </c>
       <c r="F596" s="3" t="n">
-        <v>48.18</v>
+        <v>49.23</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
       <c r="I596" s="4" t="n">
-        <v>-3.6635</v>
+        <v>-5.3262</v>
       </c>
       <c r="J596" s="4" t="n">
-        <v>-0.4897</v>
+        <v>-4.2562</v>
       </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26263,32 +26277,26 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>5.97</v>
+        <v>2.73</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.09939999999999999</v>
+        <v>0</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>35800000</v>
-      </c>
-      <c r="E597" s="8" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>142720000</v>
+      </c>
+      <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>49.23</v>
+        <v>45.93</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J597" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I597" s="6" t="inlineStr"/>
+      <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26296,7 +26304,7 @@
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26304,38 +26312,34 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>26.02</v>
+        <v>17.05</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.008399999999999999</v>
+        <v>-0.0512</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>883760</v>
-      </c>
-      <c r="E598" s="4" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>48680000</v>
+      </c>
+      <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>43.34</v>
+        <v>49.01</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="4" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26343,21 +26347,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>18.16</v>
+        <v>198.4</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0145</v>
+        <v>-0.0345</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>45490000</v>
+        <v>8520000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>52.57</v>
+        <v>61.52</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26370,7 +26374,7 @@
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26378,42 +26382,34 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>34.68</v>
+        <v>18.53</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.0181</v>
+        <v>0.0011</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>5190000</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>55440000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>43.26</v>
-      </c>
-      <c r="G600" s="3" t="n">
-        <v>13.71</v>
-      </c>
+        <v>35.89</v>
+      </c>
+      <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="4" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J600" s="4" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I600" s="2" t="inlineStr"/>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26421,23 +26417,21 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>240.1</v>
+        <v>6.06</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.02</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>10620</v>
-      </c>
-      <c r="E601" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>7340000</v>
+      </c>
+      <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>43.77</v>
+        <v>45.24</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
@@ -26445,7 +26439,7 @@
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr"/>
@@ -26454,21 +26448,21 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>2.73</v>
+        <v>77.25</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>142720000</v>
+        <v>29900000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>45.93</v>
+        <v>88.89</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26476,12 +26470,12 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26489,60 +26483,50 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>65.15000000000001</v>
+        <v>78.62</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0585</v>
+        <v>-0.0067</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>869750</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>11350000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>49.58</v>
+        <v>37.39</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
       <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="8" t="n">
-        <v>0.1431</v>
-      </c>
-      <c r="K603" s="6" t="inlineStr">
-        <is>
-          <t>Teknoloji hizmetleri</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+      <c r="J603" s="6" t="inlineStr"/>
+      <c r="K603" s="6" t="inlineStr"/>
+      <c r="L603" s="6" t="inlineStr"/>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>198.4</v>
+        <v>30.64</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0345</v>
+        <v>-0.07820000000000001</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>8520000</v>
-      </c>
-      <c r="E604" s="2" t="inlineStr"/>
+        <v>16140000</v>
+      </c>
+      <c r="E604" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F604" s="3" t="n">
-        <v>61.52</v>
+        <v>52.53</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26550,12 +26534,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26563,34 +26547,40 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>178.6</v>
+        <v>142.7</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.0341</v>
+        <v>0.061</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>8620000</v>
-      </c>
-      <c r="E605" s="6" t="inlineStr"/>
+        <v>995180</v>
+      </c>
+      <c r="E605" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F605" s="7" t="n">
-        <v>38.77</v>
+        <v>48.18</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="6" t="inlineStr"/>
-      <c r="J605" s="6" t="inlineStr"/>
+      <c r="I605" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J605" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26598,36 +26588,38 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>6.44</v>
+        <v>65.15000000000001</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.0733</v>
+        <v>-0.0585</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>19120000</v>
+        <v>869750</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.8667</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>70.31</v>
+        <v>49.58</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
       <c r="I606" s="2" t="inlineStr"/>
-      <c r="J606" s="2" t="inlineStr"/>
+      <c r="J606" s="4" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26635,21 +26627,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>18.53</v>
+        <v>42.32</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0272</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>55440000</v>
+        <v>5980000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>35.89</v>
+        <v>53.18</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26657,12 +26649,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26670,21 +26662,23 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>28.4</v>
+        <v>6.44</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>-0.0373</v>
+        <v>0.0733</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>23640000</v>
-      </c>
-      <c r="E608" s="2" t="inlineStr"/>
+        <v>19120000</v>
+      </c>
+      <c r="E608" s="4" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F608" s="3" t="n">
-        <v>55.6</v>
+        <v>70.31</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
@@ -26692,12 +26686,12 @@
       <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26705,29 +26699,35 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>6.06</v>
+        <v>9.93</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>-0.008199999999999999</v>
+        <v>0.0793</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>7340000</v>
-      </c>
-      <c r="E609" s="6" t="inlineStr"/>
+        <v>757940</v>
+      </c>
+      <c r="E609" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F609" s="7" t="n">
-        <v>45.24</v>
+        <v>61.27</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
-      <c r="I609" s="6" t="inlineStr"/>
-      <c r="J609" s="6" t="inlineStr"/>
+      <c r="I609" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J609" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr"/>
@@ -26736,35 +26736,29 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>9.93</v>
+        <v>73.8</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>0.0793</v>
+        <v>-0.0238</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>757940</v>
-      </c>
-      <c r="E610" s="4" t="n">
-        <v>0.95</v>
-      </c>
+        <v>174630</v>
+      </c>
+      <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>61.27</v>
+        <v>10.48</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
-      <c r="I610" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J610" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I610" s="2" t="inlineStr"/>
+      <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr"/>
@@ -26773,36 +26767,42 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>30.64</v>
+        <v>34.68</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.07820000000000001</v>
+        <v>-0.0181</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>16140000</v>
+        <v>5190000</v>
       </c>
       <c r="E611" s="8" t="n">
-        <v>0.2667</v>
+        <v>0.3528</v>
       </c>
       <c r="F611" s="7" t="n">
-        <v>52.53</v>
-      </c>
-      <c r="G611" s="6" t="inlineStr"/>
+        <v>43.26</v>
+      </c>
+      <c r="G611" s="7" t="n">
+        <v>13.71</v>
+      </c>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="6" t="inlineStr"/>
-      <c r="J611" s="6" t="inlineStr"/>
+      <c r="I611" s="8" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J611" s="8" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26829,7 +26829,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>19.05.2026 15:30</t>
+          <t>19.05.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 19.05.2026 17:43 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-19.xlsx
+++ b/data/bist_screener_2026-05-19.xlsx
@@ -25911,23 +25911,23 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>240.1</v>
+        <v>6.44</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.02</v>
+        <v>0.0733</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>10620</v>
+        <v>19120000</v>
       </c>
       <c r="E587" s="8" t="n">
-        <v>0.2578</v>
+        <v>0.8667</v>
       </c>
       <c r="F587" s="7" t="n">
-        <v>43.77</v>
+        <v>70.31</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25935,115 +25935,129 @@
       <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L587" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L587" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M587" s="6" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>69.09999999999999</v>
+        <v>26.02</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0162</v>
+        <v>-0.008399999999999999</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>48030</v>
+        <v>883760</v>
       </c>
       <c r="E588" s="4" t="n">
-        <v>0.58</v>
+        <v>0.9698</v>
       </c>
       <c r="F588" s="3" t="n">
-        <v>36.59</v>
+        <v>43.34</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
+      <c r="I588" s="2" t="inlineStr"/>
       <c r="J588" s="4" t="n">
-        <v>-4.155</v>
+        <v>0.6453</v>
       </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr"/>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L588" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+        </is>
+      </c>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>28.4</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0373</v>
+        <v>0.0162</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>23640000</v>
-      </c>
-      <c r="E589" s="6" t="inlineStr"/>
+        <v>48030</v>
+      </c>
+      <c r="E589" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F589" s="7" t="n">
-        <v>55.6</v>
+        <v>36.59</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="6" t="inlineStr"/>
-      <c r="J589" s="6" t="inlineStr"/>
+      <c r="I589" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J589" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr"/>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>178.6</v>
+        <v>2.48</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0341</v>
+        <v>-0.008</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>8620000</v>
-      </c>
-      <c r="E590" s="2" t="inlineStr"/>
+        <v>21880000</v>
+      </c>
+      <c r="E590" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="F590" s="3" t="n">
-        <v>38.77</v>
+        <v>35.12</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="2" t="inlineStr"/>
-      <c r="J590" s="2" t="inlineStr"/>
+      <c r="I590" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J590" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26051,38 +26065,34 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>26.02</v>
+        <v>2.73</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.008399999999999999</v>
+        <v>0</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>883760</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>142720000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>43.34</v>
+        <v>45.93</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
       <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="8" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26090,21 +26100,21 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>13.96</v>
+        <v>198.4</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0285</v>
+        <v>-0.0345</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>30370000</v>
+        <v>8520000</v>
       </c>
       <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>49.07</v>
+        <v>61.52</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26112,12 +26122,12 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26125,21 +26135,21 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>36.4</v>
+        <v>77.25</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.0196</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>6480000</v>
+        <v>29900000</v>
       </c>
       <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>58.24</v>
+        <v>88.89</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
@@ -26147,12 +26157,12 @@
       <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26160,40 +26170,34 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>2.48</v>
+        <v>13.96</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.008</v>
+        <v>-0.0285</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>21880000</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>30370000</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>35.12</v>
+        <v>49.07</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J594" s="4" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I594" s="2" t="inlineStr"/>
+      <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26201,75 +26205,71 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>18.16</v>
+        <v>9.93</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0145</v>
+        <v>0.0793</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>45490000</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
+        <v>757940</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F595" s="7" t="n">
-        <v>52.57</v>
+        <v>61.27</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="6" t="inlineStr"/>
+      <c r="I595" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J595" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr"/>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>5.97</v>
+        <v>178.6</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.09939999999999999</v>
+        <v>-0.0341</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>35800000</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>8620000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>49.23</v>
+        <v>38.77</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J596" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I596" s="2" t="inlineStr"/>
+      <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26277,21 +26277,23 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>2.73</v>
+        <v>240.1</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>142720000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>10620</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>45.93</v>
+        <v>43.77</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26299,34 +26301,32 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>17.05</v>
+        <v>30.64</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0512</v>
+        <v>-0.07820000000000001</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>48680000</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>16140000</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>49.01</v>
+        <v>52.53</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26334,12 +26334,12 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26347,56 +26347,48 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>198.4</v>
+        <v>78.62</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0345</v>
+        <v>-0.0067</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>8520000</v>
+        <v>11350000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>61.52</v>
+        <v>37.39</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
       <c r="I599" s="6" t="inlineStr"/>
       <c r="J599" s="6" t="inlineStr"/>
-      <c r="K599" s="6" t="inlineStr">
-        <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+      <c r="K599" s="6" t="inlineStr"/>
+      <c r="L599" s="6" t="inlineStr"/>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>18.53</v>
+        <v>36.4</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0011</v>
+        <v>0.0196</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>55440000</v>
+        <v>6480000</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>35.89</v>
+        <v>58.24</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26404,12 +26396,12 @@
       <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26417,21 +26409,21 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>6.06</v>
+        <v>18.53</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.008199999999999999</v>
+        <v>0.0011</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>7340000</v>
+        <v>55440000</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>45.24</v>
+        <v>35.89</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
@@ -26442,27 +26434,31 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L601" s="6" t="inlineStr"/>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>77.25</v>
+        <v>6.06</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.09960000000000001</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>29900000</v>
+        <v>7340000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>88.89</v>
+        <v>45.24</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26470,63 +26466,73 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr"/>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>78.62</v>
+        <v>34.68</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0067</v>
+        <v>-0.0181</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>11350000</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>5190000</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.3528</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>37.39</v>
-      </c>
-      <c r="G603" s="6" t="inlineStr"/>
+        <v>43.26</v>
+      </c>
+      <c r="G603" s="7" t="n">
+        <v>13.71</v>
+      </c>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="6" t="inlineStr"/>
-      <c r="K603" s="6" t="inlineStr"/>
-      <c r="L603" s="6" t="inlineStr"/>
+      <c r="I603" s="8" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J603" s="8" t="n">
+        <v>-1.4864</v>
+      </c>
+      <c r="K603" s="6" t="inlineStr">
+        <is>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>30.64</v>
+        <v>17.05</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.07820000000000001</v>
+        <v>-0.0512</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>16140000</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>48680000</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>52.53</v>
+        <v>49.01</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26534,12 +26540,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26547,79 +26553,65 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>142.7</v>
+        <v>73.8</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.061</v>
+        <v>-0.0238</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>995180</v>
-      </c>
-      <c r="E605" s="8" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>174630</v>
+      </c>
+      <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>48.18</v>
+        <v>10.48</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J605" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I605" s="6" t="inlineStr"/>
+      <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L605" s="6" t="inlineStr"/>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>65.15000000000001</v>
+        <v>18.16</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0585</v>
+        <v>0.0145</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>869750</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>45490000</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>49.58</v>
+        <v>52.57</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
       <c r="I606" s="2" t="inlineStr"/>
-      <c r="J606" s="4" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26627,21 +26619,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>42.32</v>
+        <v>28.4</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0272</v>
+        <v>-0.0373</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>5980000</v>
+        <v>23640000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>53.18</v>
+        <v>55.6</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26649,12 +26641,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26662,36 +26654,38 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>6.44</v>
+        <v>65.15000000000001</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0733</v>
+        <v>-0.0585</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>19120000</v>
+        <v>869750</v>
       </c>
       <c r="E608" s="4" t="n">
-        <v>0.8667</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F608" s="3" t="n">
-        <v>70.31</v>
+        <v>49.58</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
       <c r="I608" s="2" t="inlineStr"/>
-      <c r="J608" s="2" t="inlineStr"/>
+      <c r="J608" s="4" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26699,58 +26693,62 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>9.93</v>
+        <v>142.7</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.0793</v>
+        <v>0.061</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>757940</v>
+        <v>995180</v>
       </c>
       <c r="E609" s="8" t="n">
-        <v>0.95</v>
+        <v>0.1071</v>
       </c>
       <c r="F609" s="7" t="n">
-        <v>61.27</v>
+        <v>48.18</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
       <c r="I609" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-3.6635</v>
       </c>
       <c r="J609" s="8" t="n">
-        <v>-0.4678</v>
+        <v>-0.4897</v>
       </c>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L609" s="6" t="inlineStr"/>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L609" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M609" s="6" t="inlineStr"/>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>73.8</v>
+        <v>42.32</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.0238</v>
+        <v>0.0272</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>174630</v>
+        <v>5980000</v>
       </c>
       <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>10.48</v>
+        <v>53.18</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
@@ -26758,51 +26756,53 @@
       <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L610" s="2" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L610" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M610" s="2" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>34.68</v>
+        <v>5.97</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.0181</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>5190000</v>
+        <v>35800000</v>
       </c>
       <c r="E611" s="8" t="n">
-        <v>0.3528</v>
+        <v>0.1672</v>
       </c>
       <c r="F611" s="7" t="n">
-        <v>43.26</v>
-      </c>
-      <c r="G611" s="7" t="n">
-        <v>13.71</v>
-      </c>
+        <v>49.23</v>
+      </c>
+      <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
       <c r="I611" s="8" t="n">
-        <v>0.1029</v>
+        <v>-5.3262</v>
       </c>
       <c r="J611" s="8" t="n">
-        <v>-1.4864</v>
+        <v>-4.2562</v>
       </c>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26829,7 +26829,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>19.05.2026 16:30</t>
+          <t>19.05.2026 17:43</t>
         </is>
       </c>
     </row>

</xml_diff>